<commit_message>
cambio enlaces subida imagenes espana
</commit_message>
<xml_diff>
--- a/proyecto-monedas-2-euro-completo.xlsx
+++ b/proyecto-monedas-2-euro-completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Proyecto-euro-git\monedas-2-euro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD9D51F-EA2A-46CE-9ED9-49E28F02E9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDE3BFA-72B8-49A9-91A2-5986102D57D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5912,103 +5912,103 @@
     <t>observaciones</t>
   </si>
   <si>
-    <t>imagenes\españa-2015-cara-nacional-2euro.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2010-cara-nacional-2euro.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2002-cara-nacional-2euro.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\reverso-2eu.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2026-articulo-49.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2026-unesco-poblet.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2025-unesco-salamanca.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2024-unesco-sevilla.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2024-Policia.jpeg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2023-presidencia-ue.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2023-unesco-caceres.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2022-35-años-erasmus.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2022-elcano.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2022-unesco-garajonay.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2021-unesco-toledo.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2020-unesco-mudejar.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2019-unesco-avila.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2018-50-aniversario-felipe.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2018-unesco-santiago-compostela.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2017-unesco-naranco.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2016-unesco-segovia.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2015-30-aniversario-bandera-ue.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2015-unesco-altamira.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2014-cambio-jefatura-estado.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2014-unesco-parqueguell.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2013-unesco-escorial.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2012-diez-años-euros.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2012-unesco-burgos .jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2011-unesco-granada..jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2010-unesco-cordoba.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2009-aniversario-union-economica.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2007-tratado-roma.jpg</t>
-  </si>
-  <si>
-    <t>imagenes\españa-2005-quijote.jpg</t>
+    <t>imágenes/espana-2005-quijote.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2007-tratado-roma.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2009-aniversario-union-economica.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2010-unesco-cordoba.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2011-unesco-granada..jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2012-unesco-burgos .jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2012-diez-años-euros.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2013-unesco-escorial.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2014-unesco-parqueguell.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2014-cambio-jefatura-estado.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2015-unesco-altamira.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2015-30-aniversario-bandera-ue.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2016-unesco-segovia.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2017-unesco-naranco.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2018-unesco-santiago-compostela.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2018-50-aniversario-felipe.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2019-unesco-avila.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2020-unesco-mudejar.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2021-unesco-toledo.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2022-unesco-garajonay.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2022-elcano.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2022-35-años-erasmus.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2023-unesco-caceres.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2023-presidencia-ue.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2024-Policia.jpeg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2024-unesco-sevilla.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2025-unesco-salamanca.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2026-unesco-poblet.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2026-articulo-49.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/reverso-2eu.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2002-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2010-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imágenes/espana-2015-cara-nacional-2euro.jpg</t>
   </si>
 </sst>
 </file>
@@ -11829,7 +11829,7 @@
         <v>609</v>
       </c>
       <c r="D235" s="20" t="s">
-        <v>1864</v>
+        <v>1832</v>
       </c>
       <c r="E235" s="4" t="s">
         <v>610</v>
@@ -11853,7 +11853,7 @@
         <v>9</v>
       </c>
       <c r="D236" s="20" t="s">
-        <v>1863</v>
+        <v>1833</v>
       </c>
       <c r="E236" s="4" t="s">
         <v>10</v>
@@ -11879,7 +11879,7 @@
         <v>17</v>
       </c>
       <c r="D237" s="20" t="s">
-        <v>1862</v>
+        <v>1834</v>
       </c>
       <c r="E237" s="4" t="s">
         <v>18</v>
@@ -11905,7 +11905,7 @@
         <v>613</v>
       </c>
       <c r="D238" s="20" t="s">
-        <v>1861</v>
+        <v>1835</v>
       </c>
       <c r="E238" s="4" t="s">
         <v>614</v>
@@ -11931,7 +11931,7 @@
         <v>616</v>
       </c>
       <c r="D239" s="20" t="s">
-        <v>1860</v>
+        <v>1836</v>
       </c>
       <c r="E239" s="4" t="s">
         <v>617</v>
@@ -11957,7 +11957,7 @@
         <v>620</v>
       </c>
       <c r="D240" s="20" t="s">
-        <v>1859</v>
+        <v>1837</v>
       </c>
       <c r="E240" s="4" t="s">
         <v>621</v>
@@ -11983,7 +11983,7 @@
         <v>34</v>
       </c>
       <c r="D241" s="20" t="s">
-        <v>1858</v>
+        <v>1838</v>
       </c>
       <c r="E241" s="4" t="s">
         <v>35</v>
@@ -12009,7 +12009,7 @@
         <v>623</v>
       </c>
       <c r="D242" s="20" t="s">
-        <v>1857</v>
+        <v>1839</v>
       </c>
       <c r="E242" s="4" t="s">
         <v>624</v>
@@ -12035,7 +12035,7 @@
         <v>627</v>
       </c>
       <c r="D243" s="20" t="s">
-        <v>1856</v>
+        <v>1840</v>
       </c>
       <c r="E243" s="4" t="s">
         <v>628</v>
@@ -12061,7 +12061,7 @@
         <v>631</v>
       </c>
       <c r="D244" s="20" t="s">
-        <v>1855</v>
+        <v>1841</v>
       </c>
       <c r="E244" s="4" t="s">
         <v>632</v>
@@ -12085,7 +12085,7 @@
         <v>634</v>
       </c>
       <c r="D245" s="20" t="s">
-        <v>1854</v>
+        <v>1842</v>
       </c>
       <c r="E245" s="4" t="s">
         <v>635</v>
@@ -12111,7 +12111,7 @@
         <v>52</v>
       </c>
       <c r="D246" s="20" t="s">
-        <v>1853</v>
+        <v>1843</v>
       </c>
       <c r="E246" s="4" t="s">
         <v>638</v>
@@ -12137,7 +12137,7 @@
         <v>640</v>
       </c>
       <c r="D247" s="20" t="s">
-        <v>1852</v>
+        <v>1844</v>
       </c>
       <c r="E247" s="4" t="s">
         <v>641</v>
@@ -12163,7 +12163,7 @@
         <v>643</v>
       </c>
       <c r="D248" s="20" t="s">
-        <v>1851</v>
+        <v>1845</v>
       </c>
       <c r="E248" s="4" t="s">
         <v>644</v>
@@ -12189,7 +12189,7 @@
         <v>647</v>
       </c>
       <c r="D249" s="20" t="s">
-        <v>1850</v>
+        <v>1846</v>
       </c>
       <c r="E249" s="4" t="s">
         <v>648</v>
@@ -12215,7 +12215,7 @@
         <v>651</v>
       </c>
       <c r="D250" s="20" t="s">
-        <v>1849</v>
+        <v>1847</v>
       </c>
       <c r="E250" s="4" t="s">
         <v>652</v>
@@ -12265,7 +12265,7 @@
         <v>657</v>
       </c>
       <c r="D252" s="20" t="s">
-        <v>1847</v>
+        <v>1849</v>
       </c>
       <c r="E252" s="4" t="s">
         <v>658</v>
@@ -12291,7 +12291,7 @@
         <v>661</v>
       </c>
       <c r="D253" s="20" t="s">
-        <v>1846</v>
+        <v>1850</v>
       </c>
       <c r="E253" s="4" t="s">
         <v>662</v>
@@ -12317,7 +12317,7 @@
         <v>665</v>
       </c>
       <c r="D254" s="20" t="s">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="E254" s="4" t="s">
         <v>666</v>
@@ -12343,7 +12343,7 @@
         <v>669</v>
       </c>
       <c r="D255" s="20" t="s">
-        <v>1844</v>
+        <v>1852</v>
       </c>
       <c r="E255" s="4" t="s">
         <v>670</v>
@@ -12367,7 +12367,7 @@
         <v>84</v>
       </c>
       <c r="D256" s="20" t="s">
-        <v>1843</v>
+        <v>1853</v>
       </c>
       <c r="E256" s="4" t="s">
         <v>85</v>
@@ -12391,7 +12391,7 @@
         <v>671</v>
       </c>
       <c r="D257" s="20" t="s">
-        <v>1842</v>
+        <v>1854</v>
       </c>
       <c r="E257" s="4" t="s">
         <v>672</v>
@@ -12417,7 +12417,7 @@
         <v>675</v>
       </c>
       <c r="D258" s="20" t="s">
-        <v>1841</v>
+        <v>1855</v>
       </c>
       <c r="E258" s="4" t="s">
         <v>676</v>
@@ -12443,7 +12443,7 @@
         <v>679</v>
       </c>
       <c r="D259" s="20" t="s">
-        <v>1840</v>
+        <v>1856</v>
       </c>
       <c r="E259" s="4" t="s">
         <v>680</v>
@@ -12469,7 +12469,7 @@
         <v>682</v>
       </c>
       <c r="D260" s="20" t="s">
-        <v>1839</v>
+        <v>1857</v>
       </c>
       <c r="E260" s="4" t="s">
         <v>683</v>
@@ -12495,7 +12495,7 @@
         <v>685</v>
       </c>
       <c r="D261" s="20" t="s">
-        <v>1838</v>
+        <v>1858</v>
       </c>
       <c r="E261" s="4" t="s">
         <v>686</v>
@@ -12519,7 +12519,7 @@
         <v>688</v>
       </c>
       <c r="D262" s="20" t="s">
-        <v>1837</v>
+        <v>1859</v>
       </c>
       <c r="E262" s="4" t="s">
         <v>689</v>
@@ -12543,7 +12543,7 @@
         <v>691</v>
       </c>
       <c r="D263" s="20" t="s">
-        <v>1836</v>
+        <v>1860</v>
       </c>
       <c r="E263" s="4" t="s">
         <v>692</v>
@@ -12567,7 +12567,7 @@
         <v>694</v>
       </c>
       <c r="D264" s="20" t="s">
-        <v>1835</v>
+        <v>1861</v>
       </c>
       <c r="E264" s="4"/>
       <c r="F264" s="5"/>
@@ -12585,7 +12585,7 @@
         <v>1823</v>
       </c>
       <c r="D265" s="20" t="s">
-        <v>1834</v>
+        <v>1862</v>
       </c>
       <c r="E265" s="2" t="s">
         <v>1785</v>
@@ -12609,7 +12609,7 @@
         <v>1823</v>
       </c>
       <c r="D266" s="20" t="s">
-        <v>1833</v>
+        <v>1863</v>
       </c>
       <c r="E266" s="2" t="s">
         <v>1786</v>
@@ -12633,7 +12633,7 @@
         <v>1823</v>
       </c>
       <c r="D267" s="20" t="s">
-        <v>1832</v>
+        <v>1864</v>
       </c>
       <c r="E267" s="2" t="s">
         <v>1788</v>
@@ -25800,39 +25800,39 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D267" r:id="rId1" display="F:\Proyecto-euro-git\monedas-2-euro\imagenes\españa-2015-cara-nacional-2euro.jpg" xr:uid="{01EF2B91-067B-497D-811A-1E68C81201D9}"/>
-    <hyperlink ref="D266" r:id="rId2" xr:uid="{20DA92FC-DDAA-4683-B5DB-EC88491FC456}"/>
-    <hyperlink ref="D265" r:id="rId3" xr:uid="{E06E551E-90D6-4277-89EF-AF577122769E}"/>
-    <hyperlink ref="D264" r:id="rId4" xr:uid="{C9799AF8-AA6E-4516-907F-EA30187E55DF}"/>
-    <hyperlink ref="D263" r:id="rId5" xr:uid="{9C5CC100-196C-4D7B-8816-D8FAAF4DF726}"/>
-    <hyperlink ref="D262" r:id="rId6" xr:uid="{93645417-7D01-49C4-93C2-68D1F2E183B4}"/>
-    <hyperlink ref="D261" r:id="rId7" xr:uid="{2DE108E0-E770-4A6F-A1B1-C920462A6DCD}"/>
-    <hyperlink ref="D260" r:id="rId8" xr:uid="{C0CF5636-73D4-41BA-A68C-D313D0E6FE89}"/>
-    <hyperlink ref="D259" r:id="rId9" xr:uid="{7959D248-A790-430E-9FD9-4C33D3FDBFB7}"/>
-    <hyperlink ref="D258" r:id="rId10" xr:uid="{717745F7-B035-4148-B31F-F5050BD09573}"/>
-    <hyperlink ref="D257" r:id="rId11" xr:uid="{30123E20-DBD9-46FE-A9CF-A371EACA39A0}"/>
-    <hyperlink ref="D256" r:id="rId12" xr:uid="{6548964C-9353-4D30-9FDE-8DB56BE32FC7}"/>
-    <hyperlink ref="D255" r:id="rId13" xr:uid="{5BE091C9-B972-4E5B-AC63-7A1ED7285E6B}"/>
-    <hyperlink ref="D254" r:id="rId14" xr:uid="{F562080B-0BD1-4302-8C78-45893D4F9DBD}"/>
-    <hyperlink ref="D253" r:id="rId15" xr:uid="{F0FD06E3-113B-4663-8775-7C0C1824C5EC}"/>
-    <hyperlink ref="D252" r:id="rId16" xr:uid="{9C59C095-9458-41A0-9195-40BB5F7B3B6F}"/>
-    <hyperlink ref="D251" r:id="rId17" xr:uid="{DDB3A036-460F-4D80-A32E-0C0F0EC8C2FC}"/>
-    <hyperlink ref="D250" r:id="rId18" xr:uid="{8F7CF621-1B46-4C36-AFAC-B128C586CD5A}"/>
-    <hyperlink ref="D249" r:id="rId19" xr:uid="{A1546C6F-427C-45F6-A462-3FBA2ABF7094}"/>
-    <hyperlink ref="D248" r:id="rId20" xr:uid="{5129F731-A005-4560-95CA-71A007DCC82C}"/>
-    <hyperlink ref="D247" r:id="rId21" xr:uid="{2784F10E-0E77-42BF-B72D-E5F65DC49DF2}"/>
-    <hyperlink ref="D246" r:id="rId22" xr:uid="{159A0E30-1F76-4CC1-90D6-5B1D286AB811}"/>
-    <hyperlink ref="D245" r:id="rId23" xr:uid="{3015A5F9-84D0-49B2-80A4-77EC93B26E12}"/>
-    <hyperlink ref="D244" r:id="rId24" xr:uid="{86D4B960-E593-43BC-BE58-8358D603D613}"/>
-    <hyperlink ref="D243" r:id="rId25" xr:uid="{5EDDF15E-19F5-4BFD-8D1C-8182DEAB27DA}"/>
-    <hyperlink ref="D242" r:id="rId26" xr:uid="{C811C332-FD3A-449C-B6FC-E30702ED0682}"/>
-    <hyperlink ref="D241" r:id="rId27" xr:uid="{CDC78B92-8DB1-4AC8-826C-C2D3A08463E7}"/>
-    <hyperlink ref="D240" r:id="rId28" xr:uid="{6916C186-3284-4170-93E2-2A26EF983454}"/>
-    <hyperlink ref="D239" r:id="rId29" xr:uid="{F5FF6619-9504-40E3-9FF0-7D5A51C9DB57}"/>
-    <hyperlink ref="D238" r:id="rId30" xr:uid="{3E58B23D-AB1D-42BA-9329-4BCB6021A937}"/>
-    <hyperlink ref="D237" r:id="rId31" xr:uid="{6BE19BF0-57E9-4110-9A62-C7D279B0B62C}"/>
-    <hyperlink ref="D236" r:id="rId32" xr:uid="{A18460CF-6976-4499-B8E7-506698BA68E9}"/>
-    <hyperlink ref="D235" r:id="rId33" xr:uid="{D68F7E76-159F-4123-A05B-41142A9E7434}"/>
+    <hyperlink ref="D235" r:id="rId1" display="imagenes\espana-2005-quijote.jpg" xr:uid="{0CDEC707-9126-40FA-AC7E-B321B8776547}"/>
+    <hyperlink ref="D236" r:id="rId2" display="imagenes\espana-2007-tratado-roma.jpg" xr:uid="{DAE795C0-2816-4AFA-9F43-3004428AD845}"/>
+    <hyperlink ref="D237" r:id="rId3" display="imagenes\espana-2009-aniversario-union-economica.jpg" xr:uid="{604342E9-26F2-4F43-A925-719F63805050}"/>
+    <hyperlink ref="D265" r:id="rId4" display="imagenes\espana-2002-cara-nacional-2euro.jpg" xr:uid="{D7BFC998-9081-46E6-8509-58A5CAE8C5A5}"/>
+    <hyperlink ref="D266" r:id="rId5" display="imagenes\espana-2010-cara-nacional-2euro.jpg" xr:uid="{A927CE35-1F4F-49D0-81DC-D51200C02BE7}"/>
+    <hyperlink ref="D267" r:id="rId6" display="imagenes\espana-2015-cara-nacional-2euro.jpg" xr:uid="{196CD3B2-A69B-4537-99EA-591BF0AF933B}"/>
+    <hyperlink ref="D264" r:id="rId7" display="imagenes\reverso-2eu.jpg" xr:uid="{709BE324-7C64-4E9D-B473-404CE520A862}"/>
+    <hyperlink ref="D263" r:id="rId8" display="imagenes\espana-2026-articulo-49.jpg" xr:uid="{E8E5A1A4-B460-4DE4-BA45-13EAC4DCCE59}"/>
+    <hyperlink ref="D262" r:id="rId9" display="imagenes\espana-2026-unesco-poblet.jpg" xr:uid="{A8C73F5D-9262-4F21-A6AA-88EC7C09B60E}"/>
+    <hyperlink ref="D261" r:id="rId10" display="imagenes\espana-2025-unesco-salamanca.jpg" xr:uid="{83DB48E9-1227-4F9B-A5A1-E464FC84779A}"/>
+    <hyperlink ref="D260" r:id="rId11" display="imagenes\espana-2024-unesco-sevilla.jpg" xr:uid="{DFE97239-7C63-4443-93A2-58597CE9EF55}"/>
+    <hyperlink ref="D259" r:id="rId12" display="imagenes\espana-2024-Policia.jpeg" xr:uid="{457DF7D3-7DF9-4232-9416-D196BDBC5201}"/>
+    <hyperlink ref="D257" r:id="rId13" display="imagenes\espana-2023-unesco-caceres.jpg" xr:uid="{1CD072AE-BB3F-4B4F-8BA8-38D49A6E3B5C}"/>
+    <hyperlink ref="D258" r:id="rId14" display="imagenes\espana-2023-presidencia-ue.jpg" xr:uid="{D98778A7-627D-47AE-A4D8-4ACD59A4277D}"/>
+    <hyperlink ref="D256" r:id="rId15" display="imagenes\espana-2022-35-años-erasmus.jpg" xr:uid="{90704091-CA86-42B0-92DF-ECC7174BE57C}"/>
+    <hyperlink ref="D255" r:id="rId16" display="imagenes\espana-2022-elcano.jpg" xr:uid="{938CB225-2F3B-4582-81D1-05596FDC90B2}"/>
+    <hyperlink ref="D254" r:id="rId17" display="imagenes\espana-2022-unesco-garajonay.jpg" xr:uid="{98AB4633-DD4D-4D9F-905F-4E4082C87440}"/>
+    <hyperlink ref="D253" r:id="rId18" display="imagenes\espana-2021-unesco-toledo.jpg" xr:uid="{A99713D4-FCD5-4B56-A23B-E6DBDA880351}"/>
+    <hyperlink ref="D252" r:id="rId19" display="imagenes\espana-2020-unesco-mudejar.jpg" xr:uid="{CCBCF714-18C5-45AE-8DF1-5AC53C0C3BD4}"/>
+    <hyperlink ref="D251" r:id="rId20" display="imagenes\espana-2019-unesco-avila.jpg" xr:uid="{F55E4DED-4AC9-4816-A1A0-4D44DDDEE768}"/>
+    <hyperlink ref="D249" r:id="rId21" display="imagenes\espana-2018-unesco-santiago-compostela.jpg" xr:uid="{6039B915-F269-4012-BBEE-49DAD978D7D6}"/>
+    <hyperlink ref="D250" r:id="rId22" display="imagenes\espana-2018-50-aniversario-felipe.jpg" xr:uid="{B2B569DA-E74B-4D42-A8EF-59D700318D17}"/>
+    <hyperlink ref="D248" r:id="rId23" display="imagenes\espana-2017-unesco-naranco.jpg" xr:uid="{DE7E7CB3-0BB2-433D-9DE6-7484CC111703}"/>
+    <hyperlink ref="D247" r:id="rId24" display="imagenes\espana-2016-unesco-segovia.jpg" xr:uid="{A8EDAA71-019C-4630-8CCA-F8831D348B9A}"/>
+    <hyperlink ref="D245" r:id="rId25" display="imagenes\espana-2015-unesco-altamira.jpg" xr:uid="{57CFA499-BA67-4596-B6ED-A1562D023590}"/>
+    <hyperlink ref="D246" r:id="rId26" display="imagenes\espana-2015-30-aniversario-bandera-ue.jpg" xr:uid="{F7E123DB-0748-40BE-9A70-B20E2CA02A2C}"/>
+    <hyperlink ref="D244" r:id="rId27" display="imagenes\espana-2014-cambio-jefatura-estado.jpg" xr:uid="{29EECF9D-B1F8-44A7-BB67-E5409E09CF4D}"/>
+    <hyperlink ref="D243" r:id="rId28" display="imagenes\espana-2014-unesco-parqueguell.jpg" xr:uid="{872BE191-E05B-4826-9265-72E4593CB34A}"/>
+    <hyperlink ref="D242" r:id="rId29" display="imagenes\espana-2013-unesco-escorial.jpg" xr:uid="{3C99045C-212D-4654-B21E-AB09887C5A63}"/>
+    <hyperlink ref="D241" r:id="rId30" display="imagenes\espana-2012-diez-años-euros.jpg" xr:uid="{76652AB6-DEBD-4D5E-8339-649F1BBD247F}"/>
+    <hyperlink ref="D240" r:id="rId31" display="imagenes\espana-2012-unesco-burgos .jpg" xr:uid="{77F7290A-D8B4-4A53-B6CB-B7C4AFEE476C}"/>
+    <hyperlink ref="D239" r:id="rId32" display="imagenes\espana-2011-unesco-granada..jpg" xr:uid="{7FA02833-6422-4849-AD6F-38D1F2A3A402}"/>
+    <hyperlink ref="D238" r:id="rId33" display="imagenes\espana-2010-unesco-cordoba.jpg" xr:uid="{BEDF9C40-C842-4772-B62A-B5B23756D4A7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>

</xml_diff>

<commit_message>
arreglo enlace imagenes espana
</commit_message>
<xml_diff>
--- a/proyecto-monedas-2-euro-completo.xlsx
+++ b/proyecto-monedas-2-euro-completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Proyecto-euro-git\monedas-2-euro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDE3BFA-72B8-49A9-91A2-5986102D57D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3346B29E-E993-4101-BA8B-E8D8C33BA850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="1865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5992" uniqueCount="1865">
   <si>
     <t>Alemania</t>
   </si>
@@ -5912,103 +5912,103 @@
     <t>observaciones</t>
   </si>
   <si>
-    <t>imágenes/espana-2005-quijote.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2007-tratado-roma.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2009-aniversario-union-economica.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2010-unesco-cordoba.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2011-unesco-granada..jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2012-unesco-burgos .jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2012-diez-años-euros.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2013-unesco-escorial.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2014-unesco-parqueguell.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2014-cambio-jefatura-estado.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2015-unesco-altamira.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2015-30-aniversario-bandera-ue.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2016-unesco-segovia.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2017-unesco-naranco.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2018-unesco-santiago-compostela.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2018-50-aniversario-felipe.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2019-unesco-avila.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2020-unesco-mudejar.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2021-unesco-toledo.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2022-unesco-garajonay.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2022-elcano.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2022-35-años-erasmus.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2023-unesco-caceres.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2023-presidencia-ue.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2024-Policia.jpeg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2024-unesco-sevilla.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2025-unesco-salamanca.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2026-unesco-poblet.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2026-articulo-49.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/reverso-2eu.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2002-cara-nacional-2euro.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2010-cara-nacional-2euro.jpg</t>
-  </si>
-  <si>
-    <t>imágenes/espana-2015-cara-nacional-2euro.jpg</t>
+    <t>imagenes/espana-2005-quijote.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2007-tratado-roma.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2009-aniversario-union-economica.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2010-unesco-cordoba.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2011-unesco-granada..jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2012-unesco-burgos .jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2012-diez-años-euros.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2013-unesco-escorial.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2014-unesco-parqueguell.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2014-cambio-jefatura-estado.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2015-unesco-altamira.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2015-30-aniversario-bandera-ue.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2016-unesco-segovia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2017-unesco-naranco.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2018-unesco-santiago-compostela.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2018-50-aniversario-felipe.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2019-unesco-avila.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2020-unesco-mudejar.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2021-unesco-toledo.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2022-unesco-garajonay.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2022-elcano.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2022-35-años-erasmus.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2023-unesco-caceres.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2023-presidencia-ue.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2024-Policia.jpeg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2024-unesco-sevilla.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2025-unesco-salamanca.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2026-unesco-poblet.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2026-articulo-49.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/reverso-2eu.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2002-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2010-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/espana-2015-cara-nacional-2euro.jpg</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
subida de imagenes y enlaces alemania
</commit_message>
<xml_diff>
--- a/proyecto-monedas-2-euro-completo.xlsx
+++ b/proyecto-monedas-2-euro-completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Proyecto-euro-git\monedas-2-euro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3346B29E-E993-4101-BA8B-E8D8C33BA850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC4A34C-6CB0-4712-ACA3-00FC870DF039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5992" uniqueCount="1865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3043" uniqueCount="1908">
   <si>
     <t>Alemania</t>
   </si>
@@ -6009,6 +6009,135 @@
   </si>
   <si>
     <t>imagenes/espana-2015-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2002-cara-nacional-2euro.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2006-schleswig-holstein.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2007-pomerania-occidental.jpg</t>
+  </si>
+  <si>
+    <t>Diseño no oficial</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2007-tratado-roma.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2008-hamburgo.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2009-aniversario-union-economica.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2009-Sarre.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2010-bremen.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2011-renania-westfalia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2012-baviera.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2012-10anios-billetes-monedas-euros.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2013-tratado-eliseo.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2013-baden-wurttemberg .jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2014-baja-sajonia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2015-hesse.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2015-unidad-alemana.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2015-aniversario-bandera-ue.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2016-sajonia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2017-renania-palatinado.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2018-berlín.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2018-helmut-schmidt.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2019-bundesrat..jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2019-caida-muro-berlin.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2020-brandeburgo.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2020-arrodillamiento-varsovia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2021-sajonia-anhalt .jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2022-turingia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2022-erasmus.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2023-hamburgo.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2023-carlomagno.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2024-pomerania-occidental.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2024-constitución-paulskirche.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2025-reunificación-alemania.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2025-sarre.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2026-bremen.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2026-konrad-adenauer.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2027-renania-westfalia.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2027-dietrich-genscher.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2028-richard-von-weizsacker.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2029-annemarie-renger.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2030-helmut-kohl.jpg</t>
+  </si>
+  <si>
+    <t>imagenes/alemania-2031-regine-hildebrandt.jpg</t>
   </si>
 </sst>
 </file>
@@ -6042,12 +6171,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -6067,6 +6190,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -6089,7 +6218,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -6115,17 +6244,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -6134,20 +6260,23 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6576,7 +6705,7 @@
     <col min="3" max="3" width="118.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="29.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="94.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="29.42578125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="29.42578125" style="13" customWidth="1"/>
     <col min="7" max="7" width="19" style="1" customWidth="1"/>
     <col min="8" max="8" width="76.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="78.5703125" style="1" customWidth="1"/>
@@ -6587,28 +6716,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>1824</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>1825</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="15" t="s">
         <v>1826</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>1827</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>1828</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="18" t="s">
         <v>1829</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>1830</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="16" t="s">
         <v>1831</v>
       </c>
     </row>
@@ -6622,7 +6751,9 @@
       <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="19" t="s">
+        <v>1866</v>
+      </c>
       <c r="E2" s="4" t="s">
         <v>2</v>
       </c>
@@ -6646,7 +6777,9 @@
       <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="19" t="s">
+        <v>1867</v>
+      </c>
       <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
@@ -6670,7 +6803,9 @@
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="19" t="s">
+        <v>1869</v>
+      </c>
       <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
@@ -6694,7 +6829,9 @@
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="19" t="s">
+        <v>1870</v>
+      </c>
       <c r="E5" s="4" t="s">
         <v>14</v>
       </c>
@@ -6718,7 +6855,9 @@
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="19" t="s">
+        <v>1871</v>
+      </c>
       <c r="E6" s="4" t="s">
         <v>18</v>
       </c>
@@ -6742,7 +6881,9 @@
       <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="19" t="s">
+        <v>1872</v>
+      </c>
       <c r="E7" s="4" t="s">
         <v>21</v>
       </c>
@@ -6766,7 +6907,9 @@
       <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" s="19" t="s">
+        <v>1873</v>
+      </c>
       <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
@@ -6790,7 +6933,9 @@
       <c r="C9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" s="19" t="s">
+        <v>1874</v>
+      </c>
       <c r="E9" s="4" t="s">
         <v>29</v>
       </c>
@@ -6812,7 +6957,9 @@
       <c r="C10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" s="19" t="s">
+        <v>1875</v>
+      </c>
       <c r="E10" s="4" t="s">
         <v>32</v>
       </c>
@@ -6834,7 +6981,9 @@
       <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="2"/>
+      <c r="D11" s="19" t="s">
+        <v>1876</v>
+      </c>
       <c r="E11" s="4" t="s">
         <v>35</v>
       </c>
@@ -6858,7 +7007,9 @@
       <c r="C12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" s="19" t="s">
+        <v>1877</v>
+      </c>
       <c r="E12" s="4" t="s">
         <v>38</v>
       </c>
@@ -6882,7 +7033,9 @@
       <c r="C13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="2"/>
+      <c r="D13" s="19" t="s">
+        <v>1878</v>
+      </c>
       <c r="E13" s="4" t="s">
         <v>42</v>
       </c>
@@ -6904,7 +7057,9 @@
       <c r="C14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" s="19" t="s">
+        <v>1879</v>
+      </c>
       <c r="E14" s="4" t="s">
         <v>45</v>
       </c>
@@ -6926,7 +7081,9 @@
       <c r="C15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="19" t="s">
+        <v>1880</v>
+      </c>
       <c r="E15" s="4" t="s">
         <v>48</v>
       </c>
@@ -6948,7 +7105,9 @@
       <c r="C16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="2"/>
+      <c r="D16" s="19" t="s">
+        <v>1881</v>
+      </c>
       <c r="E16" s="4" t="s">
         <v>51</v>
       </c>
@@ -6970,7 +7129,9 @@
       <c r="C17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="2"/>
+      <c r="D17" s="19" t="s">
+        <v>1882</v>
+      </c>
       <c r="E17" s="4" t="s">
         <v>53</v>
       </c>
@@ -6994,7 +7155,9 @@
       <c r="C18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="2"/>
+      <c r="D18" s="19" t="s">
+        <v>1883</v>
+      </c>
       <c r="E18" s="4" t="s">
         <v>56</v>
       </c>
@@ -7016,7 +7179,9 @@
       <c r="C19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="2"/>
+      <c r="D19" s="19" t="s">
+        <v>1884</v>
+      </c>
       <c r="E19" s="4" t="s">
         <v>59</v>
       </c>
@@ -7038,7 +7203,9 @@
       <c r="C20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="2"/>
+      <c r="D20" s="19" t="s">
+        <v>1885</v>
+      </c>
       <c r="E20" s="4" t="s">
         <v>62</v>
       </c>
@@ -7060,7 +7227,9 @@
       <c r="C21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="2"/>
+      <c r="D21" s="19" t="s">
+        <v>1886</v>
+      </c>
       <c r="E21" s="4" t="s">
         <v>65</v>
       </c>
@@ -7082,7 +7251,9 @@
       <c r="C22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="2"/>
+      <c r="D22" s="19" t="s">
+        <v>1887</v>
+      </c>
       <c r="E22" s="4" t="s">
         <v>67</v>
       </c>
@@ -7104,7 +7275,9 @@
       <c r="C23" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D23" s="2"/>
+      <c r="D23" s="19" t="s">
+        <v>1888</v>
+      </c>
       <c r="E23" s="4" t="s">
         <v>70</v>
       </c>
@@ -7126,7 +7299,9 @@
       <c r="C24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="2"/>
+      <c r="D24" s="19" t="s">
+        <v>1889</v>
+      </c>
       <c r="E24" s="4" t="s">
         <v>73</v>
       </c>
@@ -7148,7 +7323,9 @@
       <c r="C25" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="19" t="s">
+        <v>1890</v>
+      </c>
       <c r="E25" s="4" t="s">
         <v>76</v>
       </c>
@@ -7170,7 +7347,9 @@
       <c r="C26" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D26" s="2"/>
+      <c r="D26" s="19" t="s">
+        <v>1891</v>
+      </c>
       <c r="E26" s="7" t="s">
         <v>79</v>
       </c>
@@ -7192,7 +7371,9 @@
       <c r="C27" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D27" s="2"/>
+      <c r="D27" s="19" t="s">
+        <v>1892</v>
+      </c>
       <c r="E27" s="4" t="s">
         <v>82</v>
       </c>
@@ -7214,7 +7395,9 @@
       <c r="C28" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D28" s="2"/>
+      <c r="D28" s="19" t="s">
+        <v>1893</v>
+      </c>
       <c r="E28" s="4" t="s">
         <v>85</v>
       </c>
@@ -7236,7 +7419,9 @@
       <c r="C29" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="19" t="s">
+        <v>1894</v>
+      </c>
       <c r="E29" s="4" t="s">
         <v>88</v>
       </c>
@@ -7260,7 +7445,9 @@
       <c r="C30" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D30" s="2"/>
+      <c r="D30" s="19" t="s">
+        <v>1895</v>
+      </c>
       <c r="E30" s="4" t="s">
         <v>92</v>
       </c>
@@ -7282,7 +7469,9 @@
       <c r="C31" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D31" s="2"/>
+      <c r="D31" s="19" t="s">
+        <v>1896</v>
+      </c>
       <c r="E31" s="4" t="s">
         <v>95</v>
       </c>
@@ -7306,7 +7495,9 @@
       <c r="C32" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D32" s="2"/>
+      <c r="D32" s="19" t="s">
+        <v>1897</v>
+      </c>
       <c r="E32" s="4" t="s">
         <v>99</v>
       </c>
@@ -7328,7 +7519,9 @@
       <c r="C33" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D33" s="2"/>
+      <c r="D33" s="19" t="s">
+        <v>1898</v>
+      </c>
       <c r="E33" s="4" t="s">
         <v>102</v>
       </c>
@@ -7352,7 +7545,9 @@
       <c r="C34" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D34" s="8"/>
+      <c r="D34" s="19" t="s">
+        <v>1899</v>
+      </c>
       <c r="E34" s="4" t="s">
         <v>106</v>
       </c>
@@ -7376,7 +7571,9 @@
       <c r="C35" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D35" s="2"/>
+      <c r="D35" s="19" t="s">
+        <v>1900</v>
+      </c>
       <c r="E35" s="4" t="s">
         <v>110</v>
       </c>
@@ -7398,7 +7595,9 @@
       <c r="C36" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D36" s="2"/>
+      <c r="D36" s="19" t="s">
+        <v>1901</v>
+      </c>
       <c r="E36" s="4" t="s">
         <v>113</v>
       </c>
@@ -7418,7 +7617,9 @@
       <c r="C37" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D37" s="2"/>
+      <c r="D37" s="19" t="s">
+        <v>1902</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="5"/>
       <c r="G37" s="6"/>
@@ -7434,8 +7635,12 @@
       <c r="C38" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D38" s="2"/>
-      <c r="E38" s="4"/>
+      <c r="D38" s="19" t="s">
+        <v>1903</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>1868</v>
+      </c>
       <c r="F38" s="5"/>
       <c r="G38" s="6"/>
       <c r="H38" s="2" t="s">
@@ -7452,8 +7657,12 @@
       <c r="C39" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D39" s="2"/>
-      <c r="E39" s="4"/>
+      <c r="D39" s="19" t="s">
+        <v>1904</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>1868</v>
+      </c>
       <c r="F39" s="5"/>
       <c r="G39" s="6"/>
       <c r="H39" s="2" t="s">
@@ -7470,8 +7679,12 @@
       <c r="C40" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D40" s="2"/>
-      <c r="E40" s="4"/>
+      <c r="D40" s="19" t="s">
+        <v>1905</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>1868</v>
+      </c>
       <c r="F40" s="5"/>
       <c r="G40" s="6"/>
       <c r="H40" s="2" t="s">
@@ -7488,8 +7701,12 @@
       <c r="C41" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D41" s="2"/>
-      <c r="E41" s="4"/>
+      <c r="D41" s="19" t="s">
+        <v>1906</v>
+      </c>
+      <c r="E41" s="20" t="s">
+        <v>1868</v>
+      </c>
       <c r="F41" s="5"/>
       <c r="G41" s="6"/>
       <c r="H41" s="2" t="s">
@@ -7506,8 +7723,12 @@
       <c r="C42" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="4"/>
+      <c r="D42" s="19" t="s">
+        <v>1907</v>
+      </c>
+      <c r="E42" s="20" t="s">
+        <v>1868</v>
+      </c>
       <c r="F42" s="5"/>
       <c r="G42" s="6"/>
       <c r="H42" s="2" t="s">
@@ -7521,10 +7742,12 @@
       <c r="B43" s="3">
         <v>2002</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>1823</v>
       </c>
-      <c r="D43" s="2"/>
+      <c r="D43" s="19" t="s">
+        <v>1865</v>
+      </c>
       <c r="E43" s="2" t="s">
         <v>1751</v>
       </c>
@@ -8057,7 +8280,7 @@
       <c r="B67" s="3">
         <v>2014</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D67" s="2"/>
@@ -8259,26 +8482,26 @@
       <c r="H75" s="2"/>
     </row>
     <row r="76" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="9" t="s">
+      <c r="A76" s="8" t="s">
         <v>191</v>
       </c>
       <c r="B76" s="3">
         <v>2027</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="D76" s="9"/>
-      <c r="E76" s="9" t="s">
+      <c r="D76" s="8"/>
+      <c r="E76" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="F76" s="10" t="s">
+      <c r="F76" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="G76" s="11" t="s">
+      <c r="G76" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="H76" s="9" t="s">
+      <c r="H76" s="8" t="s">
         <v>207</v>
       </c>
     </row>
@@ -8289,7 +8512,7 @@
       <c r="B77" s="3">
         <v>2002</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D77" s="2"/>
@@ -9091,50 +9314,50 @@
       </c>
     </row>
     <row r="113" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A113" s="9" t="s">
+      <c r="A113" s="8" t="s">
         <v>208</v>
       </c>
       <c r="B113" s="3">
         <v>2026</v>
       </c>
-      <c r="C113" s="9" t="s">
+      <c r="C113" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="D113" s="9"/>
-      <c r="E113" s="9" t="s">
+      <c r="D113" s="8"/>
+      <c r="E113" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="F113" s="10" t="s">
+      <c r="F113" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="G113" s="11">
+      <c r="G113" s="10">
         <v>157000</v>
       </c>
-      <c r="H113" s="9" t="s">
+      <c r="H113" s="8" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A114" s="9" t="s">
+      <c r="A114" s="8" t="s">
         <v>208</v>
       </c>
       <c r="B114" s="3">
         <v>2026</v>
       </c>
-      <c r="C114" s="9" t="s">
+      <c r="C114" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="D114" s="9"/>
-      <c r="E114" s="9" t="s">
+      <c r="D114" s="8"/>
+      <c r="E114" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="F114" s="10" t="s">
+      <c r="F114" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="G114" s="11">
+      <c r="G114" s="10">
         <v>125000</v>
       </c>
-      <c r="H114" s="9" t="s">
+      <c r="H114" s="8" t="s">
         <v>312</v>
       </c>
     </row>
@@ -9145,7 +9368,7 @@
       <c r="B115" s="3">
         <v>2002</v>
       </c>
-      <c r="C115" s="9" t="s">
+      <c r="C115" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D115" s="2"/>
@@ -9169,7 +9392,7 @@
       <c r="B116" s="3">
         <v>2008</v>
       </c>
-      <c r="C116" s="9" t="s">
+      <c r="C116" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D116" s="2"/>
@@ -9193,7 +9416,7 @@
       <c r="B117" s="3">
         <v>2009</v>
       </c>
-      <c r="C117" s="9" t="s">
+      <c r="C117" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D117" s="2"/>
@@ -9217,7 +9440,7 @@
       <c r="B118" s="3">
         <v>2014</v>
       </c>
-      <c r="C118" s="9" t="s">
+      <c r="C118" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D118" s="2"/>
@@ -9291,7 +9514,7 @@
       <c r="B122" s="3">
         <v>2026</v>
       </c>
-      <c r="C122" s="9" t="s">
+      <c r="C122" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D122" s="2"/>
@@ -9517,7 +9740,7 @@
       <c r="B132" s="3">
         <v>2008</v>
       </c>
-      <c r="C132" s="9" t="s">
+      <c r="C132" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D132" s="2"/>
@@ -10308,13 +10531,13 @@
       <c r="E167" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="F167" s="10" t="s">
+      <c r="F167" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="G167" s="11" t="s">
+      <c r="G167" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="H167" s="9" t="s">
+      <c r="H167" s="8" t="s">
         <v>442</v>
       </c>
     </row>
@@ -10325,20 +10548,20 @@
       <c r="B168" s="3">
         <v>2026</v>
       </c>
-      <c r="C168" s="12" t="s">
+      <c r="C168" s="11" t="s">
         <v>443</v>
       </c>
       <c r="D168" s="2"/>
-      <c r="E168" s="9" t="s">
+      <c r="E168" s="8" t="s">
         <v>444</v>
       </c>
-      <c r="F168" s="10" t="s">
+      <c r="F168" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="G168" s="11" t="s">
+      <c r="G168" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="H168" s="9" t="s">
+      <c r="H168" s="8" t="s">
         <v>445</v>
       </c>
     </row>
@@ -10349,7 +10572,7 @@
       <c r="B169" s="3">
         <v>2005</v>
       </c>
-      <c r="C169" s="9" t="s">
+      <c r="C169" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D169" s="2"/>
@@ -10371,7 +10594,7 @@
       <c r="B170" s="3">
         <v>2005</v>
       </c>
-      <c r="C170" s="9" t="s">
+      <c r="C170" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D170" s="2"/>
@@ -10393,7 +10616,7 @@
       <c r="B171" s="3">
         <v>2006</v>
       </c>
-      <c r="C171" s="9" t="s">
+      <c r="C171" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D171" s="2"/>
@@ -10415,7 +10638,7 @@
       <c r="B172" s="3">
         <v>2014</v>
       </c>
-      <c r="C172" s="9" t="s">
+      <c r="C172" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D172" s="2"/>
@@ -10437,7 +10660,7 @@
       <c r="B173" s="3">
         <v>2017</v>
       </c>
-      <c r="C173" s="9" t="s">
+      <c r="C173" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D173" s="2"/>
@@ -10459,7 +10682,7 @@
       <c r="B174" s="3">
         <v>2026</v>
       </c>
-      <c r="C174" s="9" t="s">
+      <c r="C174" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D174" s="2"/>
@@ -10603,16 +10826,16 @@
         <v>465</v>
       </c>
       <c r="D180" s="2"/>
-      <c r="E180" s="9" t="s">
+      <c r="E180" s="8" t="s">
         <v>466</v>
       </c>
-      <c r="F180" s="10" t="s">
+      <c r="F180" s="9" t="s">
         <v>467</v>
       </c>
       <c r="G180" s="6">
         <v>200000</v>
       </c>
-      <c r="H180" s="9" t="s">
+      <c r="H180" s="8" t="s">
         <v>468</v>
       </c>
     </row>
@@ -10647,7 +10870,7 @@
       <c r="B182" s="3">
         <v>2023</v>
       </c>
-      <c r="C182" s="9" t="s">
+      <c r="C182" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D182" s="2"/>
@@ -11247,7 +11470,7 @@
       <c r="B209" s="3">
         <v>2009</v>
       </c>
-      <c r="C209" s="9" t="s">
+      <c r="C209" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D209" s="2"/>
@@ -11803,7 +12026,7 @@
       <c r="B234" s="3">
         <v>2007</v>
       </c>
-      <c r="C234" s="9" t="s">
+      <c r="C234" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D234" s="2"/>
@@ -11828,7 +12051,7 @@
       <c r="C235" s="2" t="s">
         <v>609</v>
       </c>
-      <c r="D235" s="20" t="s">
+      <c r="D235" s="19" t="s">
         <v>1832</v>
       </c>
       <c r="E235" s="4" t="s">
@@ -11852,7 +12075,7 @@
       <c r="C236" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D236" s="20" t="s">
+      <c r="D236" s="19" t="s">
         <v>1833</v>
       </c>
       <c r="E236" s="4" t="s">
@@ -11878,7 +12101,7 @@
       <c r="C237" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D237" s="20" t="s">
+      <c r="D237" s="19" t="s">
         <v>1834</v>
       </c>
       <c r="E237" s="4" t="s">
@@ -11904,7 +12127,7 @@
       <c r="C238" s="2" t="s">
         <v>613</v>
       </c>
-      <c r="D238" s="20" t="s">
+      <c r="D238" s="19" t="s">
         <v>1835</v>
       </c>
       <c r="E238" s="4" t="s">
@@ -11930,7 +12153,7 @@
       <c r="C239" s="2" t="s">
         <v>616</v>
       </c>
-      <c r="D239" s="20" t="s">
+      <c r="D239" s="19" t="s">
         <v>1836</v>
       </c>
       <c r="E239" s="4" t="s">
@@ -11956,7 +12179,7 @@
       <c r="C240" s="2" t="s">
         <v>620</v>
       </c>
-      <c r="D240" s="20" t="s">
+      <c r="D240" s="19" t="s">
         <v>1837</v>
       </c>
       <c r="E240" s="4" t="s">
@@ -11982,7 +12205,7 @@
       <c r="C241" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D241" s="20" t="s">
+      <c r="D241" s="19" t="s">
         <v>1838</v>
       </c>
       <c r="E241" s="4" t="s">
@@ -12008,7 +12231,7 @@
       <c r="C242" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="D242" s="20" t="s">
+      <c r="D242" s="19" t="s">
         <v>1839</v>
       </c>
       <c r="E242" s="4" t="s">
@@ -12034,7 +12257,7 @@
       <c r="C243" s="2" t="s">
         <v>627</v>
       </c>
-      <c r="D243" s="20" t="s">
+      <c r="D243" s="19" t="s">
         <v>1840</v>
       </c>
       <c r="E243" s="4" t="s">
@@ -12060,7 +12283,7 @@
       <c r="C244" s="2" t="s">
         <v>631</v>
       </c>
-      <c r="D244" s="20" t="s">
+      <c r="D244" s="19" t="s">
         <v>1841</v>
       </c>
       <c r="E244" s="4" t="s">
@@ -12084,7 +12307,7 @@
       <c r="C245" s="2" t="s">
         <v>634</v>
       </c>
-      <c r="D245" s="20" t="s">
+      <c r="D245" s="19" t="s">
         <v>1842</v>
       </c>
       <c r="E245" s="4" t="s">
@@ -12110,7 +12333,7 @@
       <c r="C246" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D246" s="20" t="s">
+      <c r="D246" s="19" t="s">
         <v>1843</v>
       </c>
       <c r="E246" s="4" t="s">
@@ -12136,7 +12359,7 @@
       <c r="C247" s="2" t="s">
         <v>640</v>
       </c>
-      <c r="D247" s="20" t="s">
+      <c r="D247" s="19" t="s">
         <v>1844</v>
       </c>
       <c r="E247" s="4" t="s">
@@ -12162,7 +12385,7 @@
       <c r="C248" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="D248" s="20" t="s">
+      <c r="D248" s="19" t="s">
         <v>1845</v>
       </c>
       <c r="E248" s="4" t="s">
@@ -12188,7 +12411,7 @@
       <c r="C249" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="D249" s="20" t="s">
+      <c r="D249" s="19" t="s">
         <v>1846</v>
       </c>
       <c r="E249" s="4" t="s">
@@ -12214,7 +12437,7 @@
       <c r="C250" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="D250" s="20" t="s">
+      <c r="D250" s="19" t="s">
         <v>1847</v>
       </c>
       <c r="E250" s="4" t="s">
@@ -12238,7 +12461,7 @@
       <c r="C251" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="D251" s="20" t="s">
+      <c r="D251" s="19" t="s">
         <v>1848</v>
       </c>
       <c r="E251" s="4" t="s">
@@ -12264,7 +12487,7 @@
       <c r="C252" s="2" t="s">
         <v>657</v>
       </c>
-      <c r="D252" s="20" t="s">
+      <c r="D252" s="19" t="s">
         <v>1849</v>
       </c>
       <c r="E252" s="4" t="s">
@@ -12290,7 +12513,7 @@
       <c r="C253" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="D253" s="20" t="s">
+      <c r="D253" s="19" t="s">
         <v>1850</v>
       </c>
       <c r="E253" s="4" t="s">
@@ -12316,7 +12539,7 @@
       <c r="C254" s="2" t="s">
         <v>665</v>
       </c>
-      <c r="D254" s="20" t="s">
+      <c r="D254" s="19" t="s">
         <v>1851</v>
       </c>
       <c r="E254" s="4" t="s">
@@ -12342,7 +12565,7 @@
       <c r="C255" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="D255" s="20" t="s">
+      <c r="D255" s="19" t="s">
         <v>1852</v>
       </c>
       <c r="E255" s="4" t="s">
@@ -12366,7 +12589,7 @@
       <c r="C256" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D256" s="20" t="s">
+      <c r="D256" s="19" t="s">
         <v>1853</v>
       </c>
       <c r="E256" s="4" t="s">
@@ -12390,7 +12613,7 @@
       <c r="C257" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="D257" s="20" t="s">
+      <c r="D257" s="19" t="s">
         <v>1854</v>
       </c>
       <c r="E257" s="4" t="s">
@@ -12416,7 +12639,7 @@
       <c r="C258" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="D258" s="20" t="s">
+      <c r="D258" s="19" t="s">
         <v>1855</v>
       </c>
       <c r="E258" s="4" t="s">
@@ -12442,7 +12665,7 @@
       <c r="C259" s="2" t="s">
         <v>679</v>
       </c>
-      <c r="D259" s="20" t="s">
+      <c r="D259" s="19" t="s">
         <v>1856</v>
       </c>
       <c r="E259" s="4" t="s">
@@ -12468,7 +12691,7 @@
       <c r="C260" s="2" t="s">
         <v>682</v>
       </c>
-      <c r="D260" s="20" t="s">
+      <c r="D260" s="19" t="s">
         <v>1857</v>
       </c>
       <c r="E260" s="4" t="s">
@@ -12494,7 +12717,7 @@
       <c r="C261" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="D261" s="20" t="s">
+      <c r="D261" s="19" t="s">
         <v>1858</v>
       </c>
       <c r="E261" s="4" t="s">
@@ -12518,7 +12741,7 @@
       <c r="C262" s="2" t="s">
         <v>688</v>
       </c>
-      <c r="D262" s="20" t="s">
+      <c r="D262" s="19" t="s">
         <v>1859</v>
       </c>
       <c r="E262" s="4" t="s">
@@ -12542,7 +12765,7 @@
       <c r="C263" s="2" t="s">
         <v>691</v>
       </c>
-      <c r="D263" s="20" t="s">
+      <c r="D263" s="19" t="s">
         <v>1860</v>
       </c>
       <c r="E263" s="4" t="s">
@@ -12566,7 +12789,7 @@
       <c r="C264" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="D264" s="20" t="s">
+      <c r="D264" s="19" t="s">
         <v>1861</v>
       </c>
       <c r="E264" s="4"/>
@@ -12581,10 +12804,10 @@
       <c r="B265" s="3">
         <v>2002</v>
       </c>
-      <c r="C265" s="9" t="s">
+      <c r="C265" s="8" t="s">
         <v>1823</v>
       </c>
-      <c r="D265" s="20" t="s">
+      <c r="D265" s="19" t="s">
         <v>1862</v>
       </c>
       <c r="E265" s="2" t="s">
@@ -12605,10 +12828,10 @@
       <c r="B266" s="3">
         <v>2010</v>
       </c>
-      <c r="C266" s="9" t="s">
+      <c r="C266" s="8" t="s">
         <v>1823</v>
       </c>
-      <c r="D266" s="20" t="s">
+      <c r="D266" s="19" t="s">
         <v>1863</v>
       </c>
       <c r="E266" s="2" t="s">
@@ -12629,10 +12852,10 @@
       <c r="B267" s="3">
         <v>2015</v>
       </c>
-      <c r="C267" s="9" t="s">
+      <c r="C267" s="8" t="s">
         <v>1823</v>
       </c>
-      <c r="D267" s="20" t="s">
+      <c r="D267" s="19" t="s">
         <v>1864</v>
       </c>
       <c r="E267" s="2" t="s">
@@ -13121,7 +13344,7 @@
       <c r="B289" s="3">
         <v>2011</v>
       </c>
-      <c r="C289" s="9" t="s">
+      <c r="C289" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D289" s="2"/>
@@ -14063,7 +14286,7 @@
       <c r="B331" s="3">
         <v>2002</v>
       </c>
-      <c r="C331" s="9" t="s">
+      <c r="C331" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D331" s="2"/>
@@ -14917,7 +15140,7 @@
       <c r="B369" s="3">
         <v>2002</v>
       </c>
-      <c r="C369" s="9" t="s">
+      <c r="C369" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D369" s="2"/>
@@ -14939,7 +15162,7 @@
       <c r="B370" s="3">
         <v>2022</v>
       </c>
-      <c r="C370" s="9" t="s">
+      <c r="C370" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D370" s="2"/>
@@ -15705,7 +15928,7 @@
       <c r="B404" s="3">
         <v>2002</v>
       </c>
-      <c r="C404" s="9" t="s">
+      <c r="C404" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D404" s="2"/>
@@ -15933,26 +16156,26 @@
       </c>
     </row>
     <row r="414" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A414" s="9" t="s">
+      <c r="A414" s="8" t="s">
         <v>1050</v>
       </c>
       <c r="B414" s="3">
         <v>2026</v>
       </c>
-      <c r="C414" s="9" t="s">
+      <c r="C414" s="8" t="s">
         <v>1067</v>
       </c>
-      <c r="D414" s="9"/>
-      <c r="E414" s="13" t="s">
+      <c r="D414" s="8"/>
+      <c r="E414" s="12" t="s">
         <v>1068</v>
       </c>
-      <c r="F414" s="10" t="s">
+      <c r="F414" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="G414" s="11">
+      <c r="G414" s="10">
         <v>150000</v>
       </c>
-      <c r="H414" s="9" t="s">
+      <c r="H414" s="8" t="s">
         <v>1069</v>
       </c>
     </row>
@@ -15963,7 +16186,7 @@
       <c r="B415" s="3">
         <v>2002</v>
       </c>
-      <c r="C415" s="9" t="s">
+      <c r="C415" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D415" s="2"/>
@@ -16873,7 +17096,7 @@
       <c r="B456" s="3">
         <v>2002</v>
       </c>
-      <c r="C456" s="9" t="s">
+      <c r="C456" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D456" s="2"/>
@@ -17317,7 +17540,7 @@
       <c r="B476" s="3">
         <v>2014</v>
       </c>
-      <c r="C476" s="9" t="s">
+      <c r="C476" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D476" s="2"/>
@@ -17835,7 +18058,7 @@
       <c r="B499" s="3">
         <v>2015</v>
       </c>
-      <c r="C499" s="9" t="s">
+      <c r="C499" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D499" s="2"/>
@@ -18779,7 +19002,7 @@
       <c r="B541" s="3">
         <v>2002</v>
       </c>
-      <c r="C541" s="9" t="s">
+      <c r="C541" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D541" s="2"/>
@@ -18803,7 +19026,7 @@
       <c r="B542" s="3">
         <v>2026</v>
       </c>
-      <c r="C542" s="9" t="s">
+      <c r="C542" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D542" s="2"/>
@@ -19551,7 +19774,7 @@
       <c r="B575" s="3">
         <v>2008</v>
       </c>
-      <c r="C575" s="9" t="s">
+      <c r="C575" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D575" s="2"/>
@@ -19951,7 +20174,7 @@
       <c r="B593" s="3">
         <v>2002</v>
       </c>
-      <c r="C593" s="9" t="s">
+      <c r="C593" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D593" s="2"/>
@@ -19973,7 +20196,7 @@
       <c r="B594" s="3">
         <v>2006</v>
       </c>
-      <c r="C594" s="9" t="s">
+      <c r="C594" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D594" s="2"/>
@@ -19995,7 +20218,7 @@
       <c r="B595" s="3">
         <v>2025</v>
       </c>
-      <c r="C595" s="9" t="s">
+      <c r="C595" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D595" s="2"/>
@@ -20223,7 +20446,7 @@
       <c r="B605" s="3">
         <v>2002</v>
       </c>
-      <c r="C605" s="9" t="s">
+      <c r="C605" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D605" s="2"/>
@@ -20247,7 +20470,7 @@
       <c r="B606" s="3">
         <v>2014</v>
       </c>
-      <c r="C606" s="9" t="s">
+      <c r="C606" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D606" s="2"/>
@@ -21109,7 +21332,7 @@
       <c r="B644" s="3">
         <v>2002</v>
       </c>
-      <c r="C644" s="9" t="s">
+      <c r="C644" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D644" s="2"/>
@@ -21941,7 +22164,7 @@
       <c r="B681" s="3">
         <v>2010</v>
       </c>
-      <c r="C681" s="9" t="s">
+      <c r="C681" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D681" s="2"/>
@@ -21963,7 +22186,7 @@
       <c r="B682" s="3">
         <v>2017</v>
       </c>
-      <c r="C682" s="9" t="s">
+      <c r="C682" s="8" t="s">
         <v>1823</v>
       </c>
       <c r="D682" s="2"/>
@@ -23554,7 +23777,7 @@
       <c r="C840" s="2"/>
       <c r="D840" s="2"/>
       <c r="G840" s="2"/>
-      <c r="H840" s="15"/>
+      <c r="H840" s="14"/>
       <c r="I840" s="2"/>
       <c r="K840" s="2"/>
     </row>
@@ -23564,7 +23787,7 @@
       <c r="C841" s="2"/>
       <c r="D841" s="2"/>
       <c r="G841" s="2"/>
-      <c r="H841" s="15"/>
+      <c r="H841" s="14"/>
       <c r="I841" s="2"/>
       <c r="K841" s="2"/>
     </row>
@@ -23574,7 +23797,7 @@
       <c r="C842" s="2"/>
       <c r="D842" s="2"/>
       <c r="G842" s="2"/>
-      <c r="H842" s="15"/>
+      <c r="H842" s="14"/>
       <c r="I842" s="2"/>
       <c r="K842" s="2"/>
     </row>
@@ -23584,7 +23807,7 @@
       <c r="C843" s="2"/>
       <c r="D843" s="2"/>
       <c r="G843" s="2"/>
-      <c r="H843" s="15"/>
+      <c r="H843" s="14"/>
       <c r="I843" s="2"/>
       <c r="K843" s="2"/>
     </row>
@@ -23594,7 +23817,7 @@
       <c r="C844" s="2"/>
       <c r="D844" s="2"/>
       <c r="G844" s="2"/>
-      <c r="H844" s="15"/>
+      <c r="H844" s="14"/>
       <c r="I844" s="2"/>
       <c r="K844" s="2"/>
     </row>
@@ -23604,7 +23827,7 @@
       <c r="C845" s="2"/>
       <c r="D845" s="2"/>
       <c r="G845" s="2"/>
-      <c r="H845" s="15"/>
+      <c r="H845" s="14"/>
       <c r="I845" s="2"/>
       <c r="K845" s="2"/>
     </row>
@@ -23614,7 +23837,7 @@
       <c r="C846" s="2"/>
       <c r="D846" s="2"/>
       <c r="G846" s="2"/>
-      <c r="H846" s="15"/>
+      <c r="H846" s="14"/>
       <c r="I846" s="2"/>
       <c r="K846" s="2"/>
     </row>
@@ -23624,7 +23847,7 @@
       <c r="C847" s="2"/>
       <c r="D847" s="2"/>
       <c r="G847" s="2"/>
-      <c r="H847" s="15"/>
+      <c r="H847" s="14"/>
       <c r="I847" s="2"/>
       <c r="K847" s="2"/>
     </row>
@@ -23634,7 +23857,7 @@
       <c r="C848" s="2"/>
       <c r="D848" s="2"/>
       <c r="G848" s="2"/>
-      <c r="H848" s="15"/>
+      <c r="H848" s="14"/>
       <c r="I848" s="2"/>
       <c r="K848" s="2"/>
     </row>
@@ -23644,7 +23867,7 @@
       <c r="C849" s="2"/>
       <c r="D849" s="2"/>
       <c r="G849" s="2"/>
-      <c r="H849" s="15"/>
+      <c r="H849" s="14"/>
       <c r="I849" s="2"/>
       <c r="K849" s="2"/>
     </row>
@@ -23654,7 +23877,7 @@
       <c r="C850" s="2"/>
       <c r="D850" s="2"/>
       <c r="G850" s="2"/>
-      <c r="H850" s="15"/>
+      <c r="H850" s="14"/>
       <c r="I850" s="2"/>
       <c r="K850" s="2"/>
     </row>
@@ -23664,7 +23887,7 @@
       <c r="C851" s="2"/>
       <c r="D851" s="2"/>
       <c r="G851" s="2"/>
-      <c r="H851" s="15"/>
+      <c r="H851" s="14"/>
       <c r="I851" s="2"/>
       <c r="K851" s="2"/>
     </row>
@@ -23674,7 +23897,7 @@
       <c r="C852" s="2"/>
       <c r="D852" s="2"/>
       <c r="G852" s="2"/>
-      <c r="H852" s="15"/>
+      <c r="H852" s="14"/>
       <c r="I852" s="2"/>
       <c r="K852" s="2"/>
     </row>
@@ -23684,7 +23907,7 @@
       <c r="C853" s="2"/>
       <c r="D853" s="2"/>
       <c r="G853" s="2"/>
-      <c r="H853" s="15"/>
+      <c r="H853" s="14"/>
       <c r="I853" s="2"/>
       <c r="K853" s="2"/>
     </row>
@@ -23694,7 +23917,7 @@
       <c r="C854" s="2"/>
       <c r="D854" s="2"/>
       <c r="G854" s="2"/>
-      <c r="H854" s="15"/>
+      <c r="H854" s="14"/>
       <c r="I854" s="2"/>
       <c r="K854" s="2"/>
     </row>
@@ -23704,7 +23927,7 @@
       <c r="C855" s="2"/>
       <c r="D855" s="2"/>
       <c r="G855" s="2"/>
-      <c r="H855" s="15"/>
+      <c r="H855" s="14"/>
       <c r="I855" s="2"/>
       <c r="K855" s="2"/>
     </row>
@@ -23714,7 +23937,7 @@
       <c r="C856" s="2"/>
       <c r="D856" s="2"/>
       <c r="G856" s="2"/>
-      <c r="H856" s="15"/>
+      <c r="H856" s="14"/>
       <c r="I856" s="2"/>
       <c r="K856" s="2"/>
     </row>
@@ -23724,7 +23947,7 @@
       <c r="C857" s="2"/>
       <c r="D857" s="2"/>
       <c r="G857" s="2"/>
-      <c r="H857" s="15"/>
+      <c r="H857" s="14"/>
       <c r="I857" s="2"/>
       <c r="K857" s="2"/>
     </row>
@@ -23734,7 +23957,7 @@
       <c r="C858" s="2"/>
       <c r="D858" s="2"/>
       <c r="G858" s="2"/>
-      <c r="H858" s="15"/>
+      <c r="H858" s="14"/>
       <c r="I858" s="2"/>
       <c r="K858" s="2"/>
     </row>
@@ -23744,7 +23967,7 @@
       <c r="C859" s="2"/>
       <c r="D859" s="2"/>
       <c r="G859" s="2"/>
-      <c r="H859" s="15"/>
+      <c r="H859" s="14"/>
       <c r="I859" s="2"/>
       <c r="K859" s="2"/>
     </row>
@@ -23754,7 +23977,7 @@
       <c r="C860" s="2"/>
       <c r="D860" s="2"/>
       <c r="G860" s="2"/>
-      <c r="H860" s="15"/>
+      <c r="H860" s="14"/>
       <c r="I860" s="2"/>
       <c r="K860" s="2"/>
     </row>
@@ -23764,7 +23987,7 @@
       <c r="C861" s="2"/>
       <c r="D861" s="2"/>
       <c r="G861" s="2"/>
-      <c r="H861" s="15"/>
+      <c r="H861" s="14"/>
       <c r="I861" s="2"/>
       <c r="K861" s="2"/>
     </row>
@@ -23774,7 +23997,7 @@
       <c r="C862" s="2"/>
       <c r="D862" s="2"/>
       <c r="G862" s="2"/>
-      <c r="H862" s="15"/>
+      <c r="H862" s="14"/>
       <c r="I862" s="2"/>
       <c r="K862" s="2"/>
     </row>
@@ -23784,7 +24007,7 @@
       <c r="C863" s="2"/>
       <c r="D863" s="2"/>
       <c r="G863" s="2"/>
-      <c r="H863" s="15"/>
+      <c r="H863" s="14"/>
       <c r="I863" s="2"/>
       <c r="K863" s="2"/>
     </row>
@@ -23794,7 +24017,7 @@
       <c r="C864" s="2"/>
       <c r="D864" s="2"/>
       <c r="G864" s="2"/>
-      <c r="H864" s="15"/>
+      <c r="H864" s="14"/>
       <c r="I864" s="2"/>
       <c r="K864" s="2"/>
     </row>
@@ -23804,7 +24027,7 @@
       <c r="C865" s="2"/>
       <c r="D865" s="2"/>
       <c r="G865" s="2"/>
-      <c r="H865" s="15"/>
+      <c r="H865" s="14"/>
       <c r="I865" s="2"/>
       <c r="K865" s="2"/>
     </row>
@@ -23814,7 +24037,7 @@
       <c r="C866" s="2"/>
       <c r="D866" s="2"/>
       <c r="G866" s="2"/>
-      <c r="H866" s="15"/>
+      <c r="H866" s="14"/>
       <c r="I866" s="2"/>
       <c r="K866" s="2"/>
     </row>
@@ -23824,7 +24047,7 @@
       <c r="C867" s="2"/>
       <c r="D867" s="2"/>
       <c r="G867" s="2"/>
-      <c r="H867" s="15"/>
+      <c r="H867" s="14"/>
       <c r="I867" s="2"/>
       <c r="K867" s="2"/>
     </row>
@@ -23834,7 +24057,7 @@
       <c r="C868" s="2"/>
       <c r="D868" s="2"/>
       <c r="G868" s="2"/>
-      <c r="H868" s="15"/>
+      <c r="H868" s="14"/>
       <c r="I868" s="2"/>
       <c r="K868" s="2"/>
     </row>
@@ -23844,7 +24067,7 @@
       <c r="C869" s="2"/>
       <c r="D869" s="2"/>
       <c r="G869" s="2"/>
-      <c r="H869" s="15"/>
+      <c r="H869" s="14"/>
       <c r="I869" s="2"/>
       <c r="K869" s="2"/>
     </row>
@@ -23854,7 +24077,7 @@
       <c r="C870" s="2"/>
       <c r="D870" s="2"/>
       <c r="G870" s="2"/>
-      <c r="H870" s="15"/>
+      <c r="H870" s="14"/>
       <c r="I870" s="2"/>
       <c r="K870" s="2"/>
     </row>
@@ -23864,7 +24087,7 @@
       <c r="C871" s="2"/>
       <c r="D871" s="2"/>
       <c r="G871" s="2"/>
-      <c r="H871" s="15"/>
+      <c r="H871" s="14"/>
       <c r="I871" s="2"/>
       <c r="K871" s="2"/>
     </row>
@@ -23874,7 +24097,7 @@
       <c r="C872" s="2"/>
       <c r="D872" s="2"/>
       <c r="G872" s="2"/>
-      <c r="H872" s="15"/>
+      <c r="H872" s="14"/>
       <c r="I872" s="2"/>
       <c r="K872" s="2"/>
     </row>
@@ -23884,7 +24107,7 @@
       <c r="C873" s="2"/>
       <c r="D873" s="2"/>
       <c r="G873" s="2"/>
-      <c r="H873" s="15"/>
+      <c r="H873" s="14"/>
       <c r="I873" s="2"/>
       <c r="K873" s="2"/>
     </row>
@@ -23894,7 +24117,7 @@
       <c r="C874" s="2"/>
       <c r="D874" s="2"/>
       <c r="G874" s="2"/>
-      <c r="H874" s="15"/>
+      <c r="H874" s="14"/>
       <c r="I874" s="2"/>
       <c r="K874" s="2"/>
     </row>
@@ -23904,7 +24127,7 @@
       <c r="C875" s="2"/>
       <c r="D875" s="2"/>
       <c r="G875" s="2"/>
-      <c r="H875" s="15"/>
+      <c r="H875" s="14"/>
       <c r="I875" s="2"/>
       <c r="K875" s="2"/>
     </row>
@@ -23914,7 +24137,7 @@
       <c r="C876" s="2"/>
       <c r="D876" s="2"/>
       <c r="G876" s="2"/>
-      <c r="H876" s="15"/>
+      <c r="H876" s="14"/>
       <c r="I876" s="2"/>
       <c r="K876" s="2"/>
     </row>
@@ -23924,7 +24147,7 @@
       <c r="C877" s="2"/>
       <c r="D877" s="2"/>
       <c r="G877" s="2"/>
-      <c r="H877" s="15"/>
+      <c r="H877" s="14"/>
       <c r="I877" s="2"/>
       <c r="K877" s="2"/>
     </row>
@@ -23934,7 +24157,7 @@
       <c r="C878" s="2"/>
       <c r="D878" s="2"/>
       <c r="G878" s="2"/>
-      <c r="H878" s="15"/>
+      <c r="H878" s="14"/>
       <c r="I878" s="2"/>
       <c r="K878" s="2"/>
     </row>
@@ -23944,7 +24167,7 @@
       <c r="C879" s="2"/>
       <c r="D879" s="2"/>
       <c r="G879" s="2"/>
-      <c r="H879" s="15"/>
+      <c r="H879" s="14"/>
       <c r="I879" s="2"/>
       <c r="K879" s="2"/>
     </row>
@@ -23954,7 +24177,7 @@
       <c r="C880" s="2"/>
       <c r="D880" s="2"/>
       <c r="G880" s="2"/>
-      <c r="H880" s="15"/>
+      <c r="H880" s="14"/>
       <c r="I880" s="2"/>
       <c r="K880" s="2"/>
     </row>
@@ -23964,7 +24187,7 @@
       <c r="C881" s="2"/>
       <c r="D881" s="2"/>
       <c r="G881" s="2"/>
-      <c r="H881" s="15"/>
+      <c r="H881" s="14"/>
       <c r="I881" s="2"/>
       <c r="K881" s="2"/>
     </row>
@@ -23974,7 +24197,7 @@
       <c r="C882" s="2"/>
       <c r="D882" s="2"/>
       <c r="G882" s="2"/>
-      <c r="H882" s="15"/>
+      <c r="H882" s="14"/>
       <c r="I882" s="2"/>
       <c r="K882" s="2"/>
     </row>
@@ -23984,7 +24207,7 @@
       <c r="C883" s="2"/>
       <c r="D883" s="2"/>
       <c r="G883" s="2"/>
-      <c r="H883" s="15"/>
+      <c r="H883" s="14"/>
       <c r="I883" s="2"/>
       <c r="K883" s="2"/>
     </row>
@@ -23994,7 +24217,7 @@
       <c r="C884" s="2"/>
       <c r="D884" s="2"/>
       <c r="G884" s="2"/>
-      <c r="H884" s="15"/>
+      <c r="H884" s="14"/>
       <c r="I884" s="2"/>
       <c r="K884" s="2"/>
     </row>
@@ -24004,7 +24227,7 @@
       <c r="C885" s="2"/>
       <c r="D885" s="2"/>
       <c r="G885" s="2"/>
-      <c r="H885" s="15"/>
+      <c r="H885" s="14"/>
       <c r="I885" s="2"/>
       <c r="K885" s="2"/>
     </row>
@@ -24014,7 +24237,7 @@
       <c r="C886" s="2"/>
       <c r="D886" s="2"/>
       <c r="G886" s="2"/>
-      <c r="H886" s="15"/>
+      <c r="H886" s="14"/>
       <c r="I886" s="2"/>
       <c r="K886" s="2"/>
     </row>
@@ -24024,7 +24247,7 @@
       <c r="C887" s="2"/>
       <c r="D887" s="2"/>
       <c r="G887" s="2"/>
-      <c r="H887" s="15"/>
+      <c r="H887" s="14"/>
       <c r="I887" s="2"/>
       <c r="K887" s="2"/>
     </row>
@@ -24034,7 +24257,7 @@
       <c r="C888" s="2"/>
       <c r="D888" s="2"/>
       <c r="G888" s="2"/>
-      <c r="H888" s="15"/>
+      <c r="H888" s="14"/>
       <c r="I888" s="2"/>
       <c r="K888" s="2"/>
     </row>
@@ -24044,7 +24267,7 @@
       <c r="C889" s="2"/>
       <c r="D889" s="2"/>
       <c r="G889" s="2"/>
-      <c r="H889" s="15"/>
+      <c r="H889" s="14"/>
       <c r="I889" s="2"/>
       <c r="K889" s="2"/>
     </row>
@@ -24054,7 +24277,7 @@
       <c r="C890" s="2"/>
       <c r="D890" s="2"/>
       <c r="G890" s="2"/>
-      <c r="H890" s="15"/>
+      <c r="H890" s="14"/>
       <c r="I890" s="2"/>
       <c r="K890" s="2"/>
     </row>
@@ -24064,7 +24287,7 @@
       <c r="C891" s="2"/>
       <c r="D891" s="2"/>
       <c r="G891" s="2"/>
-      <c r="H891" s="15"/>
+      <c r="H891" s="14"/>
       <c r="I891" s="2"/>
       <c r="K891" s="2"/>
     </row>
@@ -24074,7 +24297,7 @@
       <c r="C892" s="2"/>
       <c r="D892" s="2"/>
       <c r="G892" s="2"/>
-      <c r="H892" s="15"/>
+      <c r="H892" s="14"/>
       <c r="I892" s="2"/>
       <c r="K892" s="2"/>
     </row>
@@ -24084,7 +24307,7 @@
       <c r="C893" s="2"/>
       <c r="D893" s="2"/>
       <c r="G893" s="2"/>
-      <c r="H893" s="15"/>
+      <c r="H893" s="14"/>
       <c r="I893" s="2"/>
       <c r="K893" s="2"/>
     </row>
@@ -24094,7 +24317,7 @@
       <c r="C894" s="2"/>
       <c r="D894" s="2"/>
       <c r="G894" s="2"/>
-      <c r="H894" s="15"/>
+      <c r="H894" s="14"/>
       <c r="I894" s="2"/>
       <c r="K894" s="2"/>
     </row>
@@ -24104,7 +24327,7 @@
       <c r="C895" s="2"/>
       <c r="D895" s="2"/>
       <c r="G895" s="2"/>
-      <c r="H895" s="15"/>
+      <c r="H895" s="14"/>
       <c r="I895" s="2"/>
       <c r="K895" s="2"/>
     </row>
@@ -24114,7 +24337,7 @@
       <c r="C896" s="2"/>
       <c r="D896" s="2"/>
       <c r="G896" s="2"/>
-      <c r="H896" s="15"/>
+      <c r="H896" s="14"/>
       <c r="I896" s="2"/>
       <c r="K896" s="2"/>
     </row>
@@ -24124,7 +24347,7 @@
       <c r="C897" s="2"/>
       <c r="D897" s="2"/>
       <c r="G897" s="2"/>
-      <c r="H897" s="15"/>
+      <c r="H897" s="14"/>
       <c r="I897" s="2"/>
       <c r="K897" s="2"/>
     </row>
@@ -24134,7 +24357,7 @@
       <c r="C898" s="2"/>
       <c r="D898" s="2"/>
       <c r="G898" s="2"/>
-      <c r="H898" s="15"/>
+      <c r="H898" s="14"/>
       <c r="I898" s="2"/>
       <c r="K898" s="2"/>
     </row>
@@ -24144,7 +24367,7 @@
       <c r="C899" s="2"/>
       <c r="D899" s="2"/>
       <c r="G899" s="2"/>
-      <c r="H899" s="15"/>
+      <c r="H899" s="14"/>
       <c r="I899" s="2"/>
       <c r="K899" s="2"/>
     </row>
@@ -24154,7 +24377,7 @@
       <c r="C900" s="2"/>
       <c r="D900" s="2"/>
       <c r="G900" s="2"/>
-      <c r="H900" s="15"/>
+      <c r="H900" s="14"/>
       <c r="I900" s="2"/>
       <c r="K900" s="2"/>
     </row>
@@ -24164,7 +24387,7 @@
       <c r="C901" s="2"/>
       <c r="D901" s="2"/>
       <c r="G901" s="2"/>
-      <c r="H901" s="15"/>
+      <c r="H901" s="14"/>
       <c r="I901" s="2"/>
       <c r="K901" s="2"/>
     </row>
@@ -24174,7 +24397,7 @@
       <c r="C902" s="2"/>
       <c r="D902" s="2"/>
       <c r="G902" s="2"/>
-      <c r="H902" s="15"/>
+      <c r="H902" s="14"/>
       <c r="I902" s="2"/>
       <c r="K902" s="2"/>
     </row>
@@ -24184,7 +24407,7 @@
       <c r="C903" s="2"/>
       <c r="D903" s="2"/>
       <c r="G903" s="2"/>
-      <c r="H903" s="15"/>
+      <c r="H903" s="14"/>
       <c r="I903" s="2"/>
       <c r="K903" s="2"/>
     </row>
@@ -24194,7 +24417,7 @@
       <c r="C904" s="2"/>
       <c r="D904" s="2"/>
       <c r="G904" s="2"/>
-      <c r="H904" s="15"/>
+      <c r="H904" s="14"/>
       <c r="I904" s="2"/>
       <c r="K904" s="2"/>
     </row>
@@ -24204,7 +24427,7 @@
       <c r="C905" s="2"/>
       <c r="D905" s="2"/>
       <c r="G905" s="2"/>
-      <c r="H905" s="15"/>
+      <c r="H905" s="14"/>
       <c r="I905" s="2"/>
       <c r="K905" s="2"/>
     </row>
@@ -24214,7 +24437,7 @@
       <c r="C906" s="2"/>
       <c r="D906" s="2"/>
       <c r="G906" s="2"/>
-      <c r="H906" s="15"/>
+      <c r="H906" s="14"/>
       <c r="I906" s="2"/>
       <c r="K906" s="2"/>
     </row>
@@ -24224,7 +24447,7 @@
       <c r="C907" s="2"/>
       <c r="D907" s="2"/>
       <c r="G907" s="2"/>
-      <c r="H907" s="15"/>
+      <c r="H907" s="14"/>
       <c r="I907" s="2"/>
       <c r="K907" s="2"/>
     </row>
@@ -24234,7 +24457,7 @@
       <c r="C908" s="2"/>
       <c r="D908" s="2"/>
       <c r="G908" s="2"/>
-      <c r="H908" s="15"/>
+      <c r="H908" s="14"/>
       <c r="I908" s="2"/>
       <c r="K908" s="2"/>
     </row>
@@ -24244,7 +24467,7 @@
       <c r="C909" s="2"/>
       <c r="D909" s="2"/>
       <c r="G909" s="2"/>
-      <c r="H909" s="15"/>
+      <c r="H909" s="14"/>
       <c r="I909" s="2"/>
       <c r="K909" s="2"/>
     </row>
@@ -24254,7 +24477,7 @@
       <c r="C910" s="2"/>
       <c r="D910" s="2"/>
       <c r="G910" s="2"/>
-      <c r="H910" s="15"/>
+      <c r="H910" s="14"/>
       <c r="I910" s="2"/>
       <c r="K910" s="2"/>
     </row>
@@ -24264,7 +24487,7 @@
       <c r="C911" s="2"/>
       <c r="D911" s="2"/>
       <c r="G911" s="2"/>
-      <c r="H911" s="15"/>
+      <c r="H911" s="14"/>
       <c r="I911" s="2"/>
       <c r="K911" s="2"/>
     </row>
@@ -24274,7 +24497,7 @@
       <c r="C912" s="2"/>
       <c r="D912" s="2"/>
       <c r="G912" s="2"/>
-      <c r="H912" s="15"/>
+      <c r="H912" s="14"/>
       <c r="I912" s="2"/>
       <c r="K912" s="2"/>
     </row>
@@ -24284,7 +24507,7 @@
       <c r="C913" s="2"/>
       <c r="D913" s="2"/>
       <c r="G913" s="2"/>
-      <c r="H913" s="15"/>
+      <c r="H913" s="14"/>
       <c r="I913" s="2"/>
       <c r="K913" s="2"/>
     </row>
@@ -24294,7 +24517,7 @@
       <c r="C914" s="2"/>
       <c r="D914" s="2"/>
       <c r="G914" s="2"/>
-      <c r="H914" s="15"/>
+      <c r="H914" s="14"/>
       <c r="I914" s="2"/>
       <c r="K914" s="2"/>
     </row>
@@ -24304,7 +24527,7 @@
       <c r="C915" s="2"/>
       <c r="D915" s="2"/>
       <c r="G915" s="2"/>
-      <c r="H915" s="15"/>
+      <c r="H915" s="14"/>
       <c r="I915" s="2"/>
       <c r="K915" s="2"/>
     </row>
@@ -24314,7 +24537,7 @@
       <c r="C916" s="2"/>
       <c r="D916" s="2"/>
       <c r="G916" s="2"/>
-      <c r="H916" s="15"/>
+      <c r="H916" s="14"/>
       <c r="I916" s="2"/>
       <c r="K916" s="2"/>
     </row>
@@ -24324,7 +24547,7 @@
       <c r="C917" s="2"/>
       <c r="D917" s="2"/>
       <c r="G917" s="2"/>
-      <c r="H917" s="15"/>
+      <c r="H917" s="14"/>
       <c r="I917" s="2"/>
       <c r="K917" s="2"/>
     </row>
@@ -24334,7 +24557,7 @@
       <c r="C918" s="2"/>
       <c r="D918" s="2"/>
       <c r="G918" s="2"/>
-      <c r="H918" s="15"/>
+      <c r="H918" s="14"/>
       <c r="I918" s="2"/>
       <c r="K918" s="2"/>
     </row>
@@ -24344,7 +24567,7 @@
       <c r="C919" s="2"/>
       <c r="D919" s="2"/>
       <c r="G919" s="2"/>
-      <c r="H919" s="15"/>
+      <c r="H919" s="14"/>
       <c r="I919" s="2"/>
       <c r="K919" s="2"/>
     </row>
@@ -24354,7 +24577,7 @@
       <c r="C920" s="2"/>
       <c r="D920" s="2"/>
       <c r="G920" s="2"/>
-      <c r="H920" s="15"/>
+      <c r="H920" s="14"/>
       <c r="I920" s="2"/>
       <c r="K920" s="2"/>
     </row>
@@ -24364,7 +24587,7 @@
       <c r="C921" s="2"/>
       <c r="D921" s="2"/>
       <c r="G921" s="2"/>
-      <c r="H921" s="15"/>
+      <c r="H921" s="14"/>
       <c r="I921" s="2"/>
       <c r="K921" s="2"/>
     </row>
@@ -24374,7 +24597,7 @@
       <c r="C922" s="2"/>
       <c r="D922" s="2"/>
       <c r="G922" s="2"/>
-      <c r="H922" s="15"/>
+      <c r="H922" s="14"/>
       <c r="I922" s="2"/>
       <c r="K922" s="2"/>
     </row>
@@ -24384,7 +24607,7 @@
       <c r="C923" s="2"/>
       <c r="D923" s="2"/>
       <c r="G923" s="2"/>
-      <c r="H923" s="15"/>
+      <c r="H923" s="14"/>
       <c r="I923" s="2"/>
       <c r="K923" s="2"/>
     </row>
@@ -24394,7 +24617,7 @@
       <c r="C924" s="2"/>
       <c r="D924" s="2"/>
       <c r="G924" s="2"/>
-      <c r="H924" s="15"/>
+      <c r="H924" s="14"/>
       <c r="I924" s="2"/>
       <c r="K924" s="2"/>
     </row>
@@ -24404,7 +24627,7 @@
       <c r="C925" s="2"/>
       <c r="D925" s="2"/>
       <c r="G925" s="2"/>
-      <c r="H925" s="15"/>
+      <c r="H925" s="14"/>
       <c r="I925" s="2"/>
       <c r="K925" s="2"/>
     </row>
@@ -24414,7 +24637,7 @@
       <c r="C926" s="2"/>
       <c r="D926" s="2"/>
       <c r="G926" s="2"/>
-      <c r="H926" s="15"/>
+      <c r="H926" s="14"/>
       <c r="I926" s="2"/>
       <c r="K926" s="2"/>
     </row>
@@ -24424,7 +24647,7 @@
       <c r="C927" s="2"/>
       <c r="D927" s="2"/>
       <c r="G927" s="2"/>
-      <c r="H927" s="15"/>
+      <c r="H927" s="14"/>
       <c r="I927" s="2"/>
       <c r="K927" s="2"/>
     </row>
@@ -24434,7 +24657,7 @@
       <c r="C928" s="2"/>
       <c r="D928" s="2"/>
       <c r="G928" s="2"/>
-      <c r="H928" s="15"/>
+      <c r="H928" s="14"/>
       <c r="I928" s="2"/>
       <c r="K928" s="2"/>
     </row>
@@ -24444,7 +24667,7 @@
       <c r="C929" s="2"/>
       <c r="D929" s="2"/>
       <c r="G929" s="2"/>
-      <c r="H929" s="15"/>
+      <c r="H929" s="14"/>
       <c r="I929" s="2"/>
       <c r="K929" s="2"/>
     </row>
@@ -24454,7 +24677,7 @@
       <c r="C930" s="2"/>
       <c r="D930" s="2"/>
       <c r="G930" s="2"/>
-      <c r="H930" s="15"/>
+      <c r="H930" s="14"/>
       <c r="I930" s="2"/>
       <c r="K930" s="2"/>
     </row>
@@ -24464,7 +24687,7 @@
       <c r="C931" s="2"/>
       <c r="D931" s="2"/>
       <c r="G931" s="2"/>
-      <c r="H931" s="15"/>
+      <c r="H931" s="14"/>
       <c r="I931" s="2"/>
       <c r="K931" s="2"/>
     </row>
@@ -24474,7 +24697,7 @@
       <c r="C932" s="2"/>
       <c r="D932" s="2"/>
       <c r="G932" s="2"/>
-      <c r="H932" s="15"/>
+      <c r="H932" s="14"/>
       <c r="I932" s="2"/>
       <c r="K932" s="2"/>
     </row>
@@ -24484,7 +24707,7 @@
       <c r="C933" s="2"/>
       <c r="D933" s="2"/>
       <c r="G933" s="2"/>
-      <c r="H933" s="15"/>
+      <c r="H933" s="14"/>
       <c r="I933" s="2"/>
       <c r="K933" s="2"/>
     </row>
@@ -24494,7 +24717,7 @@
       <c r="C934" s="2"/>
       <c r="D934" s="2"/>
       <c r="G934" s="2"/>
-      <c r="H934" s="15"/>
+      <c r="H934" s="14"/>
       <c r="I934" s="2"/>
       <c r="K934" s="2"/>
     </row>
@@ -24504,7 +24727,7 @@
       <c r="C935" s="2"/>
       <c r="D935" s="2"/>
       <c r="G935" s="2"/>
-      <c r="H935" s="15"/>
+      <c r="H935" s="14"/>
       <c r="I935" s="2"/>
       <c r="K935" s="2"/>
     </row>
@@ -24514,7 +24737,7 @@
       <c r="C936" s="2"/>
       <c r="D936" s="2"/>
       <c r="G936" s="2"/>
-      <c r="H936" s="15"/>
+      <c r="H936" s="14"/>
       <c r="I936" s="2"/>
       <c r="K936" s="2"/>
     </row>
@@ -24524,7 +24747,7 @@
       <c r="C937" s="2"/>
       <c r="D937" s="2"/>
       <c r="G937" s="2"/>
-      <c r="H937" s="15"/>
+      <c r="H937" s="14"/>
       <c r="I937" s="2"/>
       <c r="K937" s="2"/>
     </row>
@@ -24534,7 +24757,7 @@
       <c r="C938" s="2"/>
       <c r="D938" s="2"/>
       <c r="G938" s="2"/>
-      <c r="H938" s="15"/>
+      <c r="H938" s="14"/>
       <c r="I938" s="2"/>
       <c r="K938" s="2"/>
     </row>
@@ -24544,7 +24767,7 @@
       <c r="C939" s="2"/>
       <c r="D939" s="2"/>
       <c r="G939" s="2"/>
-      <c r="H939" s="15"/>
+      <c r="H939" s="14"/>
       <c r="I939" s="2"/>
       <c r="K939" s="2"/>
     </row>
@@ -24554,7 +24777,7 @@
       <c r="C940" s="2"/>
       <c r="D940" s="2"/>
       <c r="G940" s="2"/>
-      <c r="H940" s="15"/>
+      <c r="H940" s="14"/>
       <c r="I940" s="2"/>
       <c r="K940" s="2"/>
     </row>
@@ -24564,7 +24787,7 @@
       <c r="C941" s="2"/>
       <c r="D941" s="2"/>
       <c r="G941" s="2"/>
-      <c r="H941" s="15"/>
+      <c r="H941" s="14"/>
       <c r="I941" s="2"/>
       <c r="K941" s="2"/>
     </row>
@@ -24574,7 +24797,7 @@
       <c r="C942" s="2"/>
       <c r="D942" s="2"/>
       <c r="G942" s="2"/>
-      <c r="H942" s="15"/>
+      <c r="H942" s="14"/>
       <c r="I942" s="2"/>
       <c r="K942" s="2"/>
     </row>
@@ -24584,7 +24807,7 @@
       <c r="C943" s="2"/>
       <c r="D943" s="2"/>
       <c r="G943" s="2"/>
-      <c r="H943" s="15"/>
+      <c r="H943" s="14"/>
       <c r="I943" s="2"/>
       <c r="K943" s="2"/>
     </row>
@@ -24594,7 +24817,7 @@
       <c r="C944" s="2"/>
       <c r="D944" s="2"/>
       <c r="G944" s="2"/>
-      <c r="H944" s="15"/>
+      <c r="H944" s="14"/>
       <c r="I944" s="2"/>
       <c r="K944" s="2"/>
     </row>
@@ -24604,7 +24827,7 @@
       <c r="C945" s="2"/>
       <c r="D945" s="2"/>
       <c r="G945" s="2"/>
-      <c r="H945" s="15"/>
+      <c r="H945" s="14"/>
       <c r="I945" s="2"/>
       <c r="K945" s="2"/>
     </row>
@@ -24614,7 +24837,7 @@
       <c r="C946" s="2"/>
       <c r="D946" s="2"/>
       <c r="G946" s="2"/>
-      <c r="H946" s="15"/>
+      <c r="H946" s="14"/>
       <c r="I946" s="2"/>
       <c r="K946" s="2"/>
     </row>
@@ -24624,7 +24847,7 @@
       <c r="C947" s="2"/>
       <c r="D947" s="2"/>
       <c r="G947" s="2"/>
-      <c r="H947" s="15"/>
+      <c r="H947" s="14"/>
       <c r="I947" s="2"/>
       <c r="K947" s="2"/>
     </row>
@@ -24634,7 +24857,7 @@
       <c r="C948" s="2"/>
       <c r="D948" s="2"/>
       <c r="G948" s="2"/>
-      <c r="H948" s="15"/>
+      <c r="H948" s="14"/>
       <c r="I948" s="2"/>
       <c r="K948" s="2"/>
     </row>
@@ -24644,7 +24867,7 @@
       <c r="C949" s="2"/>
       <c r="D949" s="2"/>
       <c r="G949" s="2"/>
-      <c r="H949" s="15"/>
+      <c r="H949" s="14"/>
       <c r="I949" s="2"/>
       <c r="K949" s="2"/>
     </row>
@@ -24654,7 +24877,7 @@
       <c r="C950" s="2"/>
       <c r="D950" s="2"/>
       <c r="G950" s="2"/>
-      <c r="H950" s="15"/>
+      <c r="H950" s="14"/>
       <c r="I950" s="2"/>
       <c r="K950" s="2"/>
     </row>
@@ -24664,7 +24887,7 @@
       <c r="C951" s="2"/>
       <c r="D951" s="2"/>
       <c r="G951" s="2"/>
-      <c r="H951" s="15"/>
+      <c r="H951" s="14"/>
       <c r="I951" s="2"/>
       <c r="K951" s="2"/>
     </row>
@@ -24674,7 +24897,7 @@
       <c r="C952" s="2"/>
       <c r="D952" s="2"/>
       <c r="G952" s="2"/>
-      <c r="H952" s="15"/>
+      <c r="H952" s="14"/>
       <c r="I952" s="2"/>
       <c r="K952" s="2"/>
     </row>
@@ -24684,7 +24907,7 @@
       <c r="C953" s="2"/>
       <c r="D953" s="2"/>
       <c r="G953" s="2"/>
-      <c r="H953" s="15"/>
+      <c r="H953" s="14"/>
       <c r="I953" s="2"/>
       <c r="K953" s="2"/>
     </row>
@@ -24694,7 +24917,7 @@
       <c r="C954" s="2"/>
       <c r="D954" s="2"/>
       <c r="G954" s="2"/>
-      <c r="H954" s="15"/>
+      <c r="H954" s="14"/>
       <c r="I954" s="2"/>
       <c r="K954" s="2"/>
     </row>
@@ -24704,7 +24927,7 @@
       <c r="C955" s="2"/>
       <c r="D955" s="2"/>
       <c r="G955" s="2"/>
-      <c r="H955" s="15"/>
+      <c r="H955" s="14"/>
       <c r="I955" s="2"/>
       <c r="K955" s="2"/>
     </row>
@@ -24714,7 +24937,7 @@
       <c r="C956" s="2"/>
       <c r="D956" s="2"/>
       <c r="G956" s="2"/>
-      <c r="H956" s="15"/>
+      <c r="H956" s="14"/>
       <c r="I956" s="2"/>
       <c r="K956" s="2"/>
     </row>
@@ -24724,7 +24947,7 @@
       <c r="C957" s="2"/>
       <c r="D957" s="2"/>
       <c r="G957" s="2"/>
-      <c r="H957" s="15"/>
+      <c r="H957" s="14"/>
       <c r="I957" s="2"/>
       <c r="K957" s="2"/>
     </row>
@@ -24734,7 +24957,7 @@
       <c r="C958" s="2"/>
       <c r="D958" s="2"/>
       <c r="G958" s="2"/>
-      <c r="H958" s="15"/>
+      <c r="H958" s="14"/>
       <c r="I958" s="2"/>
       <c r="K958" s="2"/>
     </row>
@@ -24744,7 +24967,7 @@
       <c r="C959" s="2"/>
       <c r="D959" s="2"/>
       <c r="G959" s="2"/>
-      <c r="H959" s="15"/>
+      <c r="H959" s="14"/>
       <c r="I959" s="2"/>
       <c r="K959" s="2"/>
     </row>
@@ -24754,7 +24977,7 @@
       <c r="C960" s="2"/>
       <c r="D960" s="2"/>
       <c r="G960" s="2"/>
-      <c r="H960" s="15"/>
+      <c r="H960" s="14"/>
       <c r="I960" s="2"/>
       <c r="K960" s="2"/>
     </row>
@@ -24764,7 +24987,7 @@
       <c r="C961" s="2"/>
       <c r="D961" s="2"/>
       <c r="G961" s="2"/>
-      <c r="H961" s="15"/>
+      <c r="H961" s="14"/>
       <c r="I961" s="2"/>
       <c r="K961" s="2"/>
     </row>
@@ -24774,7 +24997,7 @@
       <c r="C962" s="2"/>
       <c r="D962" s="2"/>
       <c r="G962" s="2"/>
-      <c r="H962" s="15"/>
+      <c r="H962" s="14"/>
       <c r="I962" s="2"/>
       <c r="K962" s="2"/>
     </row>
@@ -24784,7 +25007,7 @@
       <c r="C963" s="2"/>
       <c r="D963" s="2"/>
       <c r="G963" s="2"/>
-      <c r="H963" s="15"/>
+      <c r="H963" s="14"/>
       <c r="I963" s="2"/>
       <c r="K963" s="2"/>
     </row>
@@ -24794,7 +25017,7 @@
       <c r="C964" s="2"/>
       <c r="D964" s="2"/>
       <c r="G964" s="2"/>
-      <c r="H964" s="15"/>
+      <c r="H964" s="14"/>
       <c r="I964" s="2"/>
       <c r="K964" s="2"/>
     </row>
@@ -24804,7 +25027,7 @@
       <c r="C965" s="2"/>
       <c r="D965" s="2"/>
       <c r="G965" s="2"/>
-      <c r="H965" s="15"/>
+      <c r="H965" s="14"/>
       <c r="I965" s="2"/>
       <c r="K965" s="2"/>
     </row>
@@ -24814,7 +25037,7 @@
       <c r="C966" s="2"/>
       <c r="D966" s="2"/>
       <c r="G966" s="2"/>
-      <c r="H966" s="15"/>
+      <c r="H966" s="14"/>
       <c r="I966" s="2"/>
       <c r="K966" s="2"/>
     </row>
@@ -24824,7 +25047,7 @@
       <c r="C967" s="2"/>
       <c r="D967" s="2"/>
       <c r="G967" s="2"/>
-      <c r="H967" s="15"/>
+      <c r="H967" s="14"/>
       <c r="I967" s="2"/>
       <c r="K967" s="2"/>
     </row>
@@ -24834,7 +25057,7 @@
       <c r="C968" s="2"/>
       <c r="D968" s="2"/>
       <c r="G968" s="2"/>
-      <c r="H968" s="15"/>
+      <c r="H968" s="14"/>
       <c r="I968" s="2"/>
       <c r="K968" s="2"/>
     </row>
@@ -24844,7 +25067,7 @@
       <c r="C969" s="2"/>
       <c r="D969" s="2"/>
       <c r="G969" s="2"/>
-      <c r="H969" s="15"/>
+      <c r="H969" s="14"/>
       <c r="I969" s="2"/>
       <c r="K969" s="2"/>
     </row>
@@ -24854,7 +25077,7 @@
       <c r="C970" s="2"/>
       <c r="D970" s="2"/>
       <c r="G970" s="2"/>
-      <c r="H970" s="15"/>
+      <c r="H970" s="14"/>
       <c r="I970" s="2"/>
       <c r="K970" s="2"/>
     </row>
@@ -24864,7 +25087,7 @@
       <c r="C971" s="2"/>
       <c r="D971" s="2"/>
       <c r="G971" s="2"/>
-      <c r="H971" s="15"/>
+      <c r="H971" s="14"/>
       <c r="I971" s="2"/>
       <c r="K971" s="2"/>
     </row>
@@ -24874,7 +25097,7 @@
       <c r="C972" s="2"/>
       <c r="D972" s="2"/>
       <c r="G972" s="2"/>
-      <c r="H972" s="15"/>
+      <c r="H972" s="14"/>
       <c r="I972" s="2"/>
       <c r="K972" s="2"/>
     </row>
@@ -24884,7 +25107,7 @@
       <c r="C973" s="2"/>
       <c r="D973" s="2"/>
       <c r="G973" s="2"/>
-      <c r="H973" s="15"/>
+      <c r="H973" s="14"/>
       <c r="I973" s="2"/>
       <c r="K973" s="2"/>
     </row>
@@ -24894,7 +25117,7 @@
       <c r="C974" s="2"/>
       <c r="D974" s="2"/>
       <c r="G974" s="2"/>
-      <c r="H974" s="15"/>
+      <c r="H974" s="14"/>
       <c r="I974" s="2"/>
       <c r="K974" s="2"/>
     </row>
@@ -24904,7 +25127,7 @@
       <c r="C975" s="2"/>
       <c r="D975" s="2"/>
       <c r="G975" s="2"/>
-      <c r="H975" s="15"/>
+      <c r="H975" s="14"/>
       <c r="I975" s="2"/>
       <c r="K975" s="2"/>
     </row>
@@ -24914,7 +25137,7 @@
       <c r="C976" s="2"/>
       <c r="D976" s="2"/>
       <c r="G976" s="2"/>
-      <c r="H976" s="15"/>
+      <c r="H976" s="14"/>
       <c r="I976" s="2"/>
       <c r="K976" s="2"/>
     </row>
@@ -24924,7 +25147,7 @@
       <c r="C977" s="2"/>
       <c r="D977" s="2"/>
       <c r="G977" s="2"/>
-      <c r="H977" s="15"/>
+      <c r="H977" s="14"/>
       <c r="I977" s="2"/>
       <c r="K977" s="2"/>
     </row>
@@ -24934,7 +25157,7 @@
       <c r="C978" s="2"/>
       <c r="D978" s="2"/>
       <c r="G978" s="2"/>
-      <c r="H978" s="15"/>
+      <c r="H978" s="14"/>
       <c r="I978" s="2"/>
       <c r="K978" s="2"/>
     </row>
@@ -24944,7 +25167,7 @@
       <c r="C979" s="2"/>
       <c r="D979" s="2"/>
       <c r="G979" s="2"/>
-      <c r="H979" s="15"/>
+      <c r="H979" s="14"/>
       <c r="I979" s="2"/>
       <c r="K979" s="2"/>
     </row>
@@ -24954,7 +25177,7 @@
       <c r="C980" s="2"/>
       <c r="D980" s="2"/>
       <c r="G980" s="2"/>
-      <c r="H980" s="15"/>
+      <c r="H980" s="14"/>
       <c r="I980" s="2"/>
       <c r="K980" s="2"/>
     </row>
@@ -24964,7 +25187,7 @@
       <c r="C981" s="2"/>
       <c r="D981" s="2"/>
       <c r="G981" s="2"/>
-      <c r="H981" s="15"/>
+      <c r="H981" s="14"/>
       <c r="I981" s="2"/>
       <c r="K981" s="2"/>
     </row>
@@ -24974,7 +25197,7 @@
       <c r="C982" s="2"/>
       <c r="D982" s="2"/>
       <c r="G982" s="2"/>
-      <c r="H982" s="15"/>
+      <c r="H982" s="14"/>
       <c r="I982" s="2"/>
       <c r="K982" s="2"/>
     </row>
@@ -24984,7 +25207,7 @@
       <c r="C983" s="2"/>
       <c r="D983" s="2"/>
       <c r="G983" s="2"/>
-      <c r="H983" s="15"/>
+      <c r="H983" s="14"/>
       <c r="I983" s="2"/>
       <c r="K983" s="2"/>
     </row>
@@ -24994,7 +25217,7 @@
       <c r="C984" s="2"/>
       <c r="D984" s="2"/>
       <c r="G984" s="2"/>
-      <c r="H984" s="15"/>
+      <c r="H984" s="14"/>
       <c r="I984" s="2"/>
       <c r="K984" s="2"/>
     </row>
@@ -25004,7 +25227,7 @@
       <c r="C985" s="2"/>
       <c r="D985" s="2"/>
       <c r="G985" s="2"/>
-      <c r="H985" s="15"/>
+      <c r="H985" s="14"/>
       <c r="I985" s="2"/>
       <c r="K985" s="2"/>
     </row>
@@ -25014,7 +25237,7 @@
       <c r="C986" s="2"/>
       <c r="D986" s="2"/>
       <c r="G986" s="2"/>
-      <c r="H986" s="15"/>
+      <c r="H986" s="14"/>
       <c r="I986" s="2"/>
       <c r="K986" s="2"/>
     </row>
@@ -25024,7 +25247,7 @@
       <c r="C987" s="2"/>
       <c r="D987" s="2"/>
       <c r="G987" s="2"/>
-      <c r="H987" s="15"/>
+      <c r="H987" s="14"/>
       <c r="I987" s="2"/>
       <c r="K987" s="2"/>
     </row>
@@ -25034,7 +25257,7 @@
       <c r="C988" s="2"/>
       <c r="D988" s="2"/>
       <c r="G988" s="2"/>
-      <c r="H988" s="15"/>
+      <c r="H988" s="14"/>
       <c r="I988" s="2"/>
       <c r="K988" s="2"/>
     </row>
@@ -25044,7 +25267,7 @@
       <c r="C989" s="2"/>
       <c r="D989" s="2"/>
       <c r="G989" s="2"/>
-      <c r="H989" s="15"/>
+      <c r="H989" s="14"/>
       <c r="I989" s="2"/>
       <c r="K989" s="2"/>
     </row>
@@ -25054,7 +25277,7 @@
       <c r="C990" s="2"/>
       <c r="D990" s="2"/>
       <c r="G990" s="2"/>
-      <c r="H990" s="15"/>
+      <c r="H990" s="14"/>
       <c r="I990" s="2"/>
       <c r="K990" s="2"/>
     </row>
@@ -25064,7 +25287,7 @@
       <c r="C991" s="2"/>
       <c r="D991" s="2"/>
       <c r="G991" s="2"/>
-      <c r="H991" s="15"/>
+      <c r="H991" s="14"/>
       <c r="I991" s="2"/>
       <c r="K991" s="2"/>
     </row>
@@ -25074,7 +25297,7 @@
       <c r="C992" s="2"/>
       <c r="D992" s="2"/>
       <c r="G992" s="2"/>
-      <c r="H992" s="15"/>
+      <c r="H992" s="14"/>
       <c r="I992" s="2"/>
       <c r="K992" s="2"/>
     </row>
@@ -25084,7 +25307,7 @@
       <c r="C993" s="2"/>
       <c r="D993" s="2"/>
       <c r="G993" s="2"/>
-      <c r="H993" s="15"/>
+      <c r="H993" s="14"/>
       <c r="I993" s="2"/>
       <c r="K993" s="2"/>
     </row>
@@ -25094,7 +25317,7 @@
       <c r="C994" s="2"/>
       <c r="D994" s="2"/>
       <c r="G994" s="2"/>
-      <c r="H994" s="15"/>
+      <c r="H994" s="14"/>
       <c r="I994" s="2"/>
       <c r="K994" s="2"/>
     </row>
@@ -25104,7 +25327,7 @@
       <c r="C995" s="2"/>
       <c r="D995" s="2"/>
       <c r="G995" s="2"/>
-      <c r="H995" s="15"/>
+      <c r="H995" s="14"/>
       <c r="I995" s="2"/>
       <c r="K995" s="2"/>
     </row>
@@ -25114,7 +25337,7 @@
       <c r="C996" s="2"/>
       <c r="D996" s="2"/>
       <c r="G996" s="2"/>
-      <c r="H996" s="15"/>
+      <c r="H996" s="14"/>
       <c r="I996" s="2"/>
       <c r="K996" s="2"/>
     </row>
@@ -25124,7 +25347,7 @@
       <c r="C997" s="2"/>
       <c r="D997" s="2"/>
       <c r="G997" s="2"/>
-      <c r="H997" s="15"/>
+      <c r="H997" s="14"/>
       <c r="I997" s="2"/>
       <c r="K997" s="2"/>
     </row>
@@ -25134,7 +25357,7 @@
       <c r="C998" s="2"/>
       <c r="D998" s="2"/>
       <c r="G998" s="2"/>
-      <c r="H998" s="15"/>
+      <c r="H998" s="14"/>
       <c r="I998" s="2"/>
       <c r="K998" s="2"/>
     </row>
@@ -25144,7 +25367,7 @@
       <c r="C999" s="2"/>
       <c r="D999" s="2"/>
       <c r="G999" s="2"/>
-      <c r="H999" s="15"/>
+      <c r="H999" s="14"/>
       <c r="I999" s="2"/>
       <c r="K999" s="2"/>
     </row>
@@ -25154,7 +25377,7 @@
       <c r="C1000" s="2"/>
       <c r="D1000" s="2"/>
       <c r="G1000" s="2"/>
-      <c r="H1000" s="15"/>
+      <c r="H1000" s="14"/>
       <c r="I1000" s="2"/>
       <c r="K1000" s="2"/>
     </row>
@@ -25164,7 +25387,7 @@
       <c r="C1001" s="2"/>
       <c r="D1001" s="2"/>
       <c r="G1001" s="2"/>
-      <c r="H1001" s="15"/>
+      <c r="H1001" s="14"/>
       <c r="I1001" s="2"/>
       <c r="K1001" s="2"/>
     </row>
@@ -25174,7 +25397,7 @@
       <c r="C1002" s="2"/>
       <c r="D1002" s="2"/>
       <c r="G1002" s="2"/>
-      <c r="H1002" s="15"/>
+      <c r="H1002" s="14"/>
       <c r="I1002" s="2"/>
       <c r="K1002" s="2"/>
     </row>
@@ -25184,7 +25407,7 @@
       <c r="C1003" s="2"/>
       <c r="D1003" s="2"/>
       <c r="G1003" s="2"/>
-      <c r="H1003" s="15"/>
+      <c r="H1003" s="14"/>
       <c r="I1003" s="2"/>
       <c r="K1003" s="2"/>
     </row>
@@ -25194,7 +25417,7 @@
       <c r="C1004" s="2"/>
       <c r="D1004" s="2"/>
       <c r="G1004" s="2"/>
-      <c r="H1004" s="15"/>
+      <c r="H1004" s="14"/>
       <c r="I1004" s="2"/>
       <c r="K1004" s="2"/>
     </row>
@@ -25204,7 +25427,7 @@
       <c r="C1005" s="2"/>
       <c r="D1005" s="2"/>
       <c r="G1005" s="2"/>
-      <c r="H1005" s="15"/>
+      <c r="H1005" s="14"/>
       <c r="I1005" s="2"/>
       <c r="K1005" s="2"/>
     </row>
@@ -25214,7 +25437,7 @@
       <c r="C1006" s="2"/>
       <c r="D1006" s="2"/>
       <c r="G1006" s="2"/>
-      <c r="H1006" s="15"/>
+      <c r="H1006" s="14"/>
       <c r="I1006" s="2"/>
       <c r="K1006" s="2"/>
     </row>
@@ -25224,7 +25447,7 @@
       <c r="C1007" s="2"/>
       <c r="D1007" s="2"/>
       <c r="G1007" s="2"/>
-      <c r="H1007" s="15"/>
+      <c r="H1007" s="14"/>
       <c r="I1007" s="2"/>
       <c r="K1007" s="2"/>
     </row>
@@ -25234,7 +25457,7 @@
       <c r="C1008" s="2"/>
       <c r="D1008" s="2"/>
       <c r="G1008" s="2"/>
-      <c r="H1008" s="15"/>
+      <c r="H1008" s="14"/>
       <c r="I1008" s="2"/>
       <c r="K1008" s="2"/>
     </row>
@@ -25244,7 +25467,7 @@
       <c r="C1009" s="2"/>
       <c r="D1009" s="2"/>
       <c r="G1009" s="2"/>
-      <c r="H1009" s="15"/>
+      <c r="H1009" s="14"/>
       <c r="I1009" s="2"/>
       <c r="K1009" s="2"/>
     </row>
@@ -25254,7 +25477,7 @@
       <c r="C1010" s="2"/>
       <c r="D1010" s="2"/>
       <c r="G1010" s="2"/>
-      <c r="H1010" s="15"/>
+      <c r="H1010" s="14"/>
       <c r="I1010" s="2"/>
       <c r="K1010" s="2"/>
     </row>
@@ -25264,7 +25487,7 @@
       <c r="C1011" s="2"/>
       <c r="D1011" s="2"/>
       <c r="G1011" s="2"/>
-      <c r="H1011" s="15"/>
+      <c r="H1011" s="14"/>
       <c r="I1011" s="2"/>
       <c r="K1011" s="2"/>
     </row>
@@ -25274,7 +25497,7 @@
       <c r="C1012" s="2"/>
       <c r="D1012" s="2"/>
       <c r="G1012" s="2"/>
-      <c r="H1012" s="15"/>
+      <c r="H1012" s="14"/>
       <c r="I1012" s="2"/>
       <c r="K1012" s="2"/>
     </row>
@@ -25284,7 +25507,7 @@
       <c r="C1013" s="2"/>
       <c r="D1013" s="2"/>
       <c r="G1013" s="2"/>
-      <c r="H1013" s="15"/>
+      <c r="H1013" s="14"/>
       <c r="I1013" s="2"/>
       <c r="K1013" s="2"/>
     </row>
@@ -25294,7 +25517,7 @@
       <c r="C1014" s="2"/>
       <c r="D1014" s="2"/>
       <c r="G1014" s="2"/>
-      <c r="H1014" s="15"/>
+      <c r="H1014" s="14"/>
       <c r="I1014" s="2"/>
       <c r="K1014" s="2"/>
     </row>
@@ -25304,7 +25527,7 @@
       <c r="C1015" s="2"/>
       <c r="D1015" s="2"/>
       <c r="G1015" s="2"/>
-      <c r="H1015" s="15"/>
+      <c r="H1015" s="14"/>
       <c r="I1015" s="2"/>
       <c r="K1015" s="2"/>
     </row>
@@ -25314,7 +25537,7 @@
       <c r="C1016" s="2"/>
       <c r="D1016" s="2"/>
       <c r="G1016" s="2"/>
-      <c r="H1016" s="15"/>
+      <c r="H1016" s="14"/>
       <c r="I1016" s="2"/>
       <c r="K1016" s="2"/>
     </row>
@@ -25324,7 +25547,7 @@
       <c r="C1017" s="2"/>
       <c r="D1017" s="2"/>
       <c r="G1017" s="2"/>
-      <c r="H1017" s="15"/>
+      <c r="H1017" s="14"/>
       <c r="I1017" s="2"/>
       <c r="K1017" s="2"/>
     </row>
@@ -25334,7 +25557,7 @@
       <c r="C1018" s="2"/>
       <c r="D1018" s="2"/>
       <c r="G1018" s="2"/>
-      <c r="H1018" s="15"/>
+      <c r="H1018" s="14"/>
       <c r="I1018" s="2"/>
       <c r="K1018" s="2"/>
     </row>
@@ -25344,7 +25567,7 @@
       <c r="C1019" s="2"/>
       <c r="D1019" s="2"/>
       <c r="G1019" s="2"/>
-      <c r="H1019" s="15"/>
+      <c r="H1019" s="14"/>
       <c r="I1019" s="2"/>
       <c r="K1019" s="2"/>
     </row>
@@ -25354,7 +25577,7 @@
       <c r="C1020" s="2"/>
       <c r="D1020" s="2"/>
       <c r="G1020" s="2"/>
-      <c r="H1020" s="15"/>
+      <c r="H1020" s="14"/>
       <c r="I1020" s="2"/>
       <c r="K1020" s="2"/>
     </row>
@@ -25364,7 +25587,7 @@
       <c r="C1021" s="2"/>
       <c r="D1021" s="2"/>
       <c r="G1021" s="2"/>
-      <c r="H1021" s="15"/>
+      <c r="H1021" s="14"/>
       <c r="I1021" s="2"/>
       <c r="K1021" s="2"/>
     </row>
@@ -25374,7 +25597,7 @@
       <c r="C1022" s="2"/>
       <c r="D1022" s="2"/>
       <c r="G1022" s="2"/>
-      <c r="H1022" s="15"/>
+      <c r="H1022" s="14"/>
       <c r="I1022" s="2"/>
       <c r="K1022" s="2"/>
     </row>
@@ -25384,7 +25607,7 @@
       <c r="C1023" s="2"/>
       <c r="D1023" s="2"/>
       <c r="G1023" s="2"/>
-      <c r="H1023" s="15"/>
+      <c r="H1023" s="14"/>
       <c r="I1023" s="2"/>
       <c r="K1023" s="2"/>
     </row>
@@ -25394,7 +25617,7 @@
       <c r="C1024" s="2"/>
       <c r="D1024" s="2"/>
       <c r="G1024" s="2"/>
-      <c r="H1024" s="15"/>
+      <c r="H1024" s="14"/>
       <c r="I1024" s="2"/>
       <c r="K1024" s="2"/>
     </row>
@@ -25404,7 +25627,7 @@
       <c r="C1025" s="2"/>
       <c r="D1025" s="2"/>
       <c r="G1025" s="2"/>
-      <c r="H1025" s="15"/>
+      <c r="H1025" s="14"/>
       <c r="I1025" s="2"/>
       <c r="K1025" s="2"/>
     </row>
@@ -25414,7 +25637,7 @@
       <c r="C1026" s="2"/>
       <c r="D1026" s="2"/>
       <c r="G1026" s="2"/>
-      <c r="H1026" s="15"/>
+      <c r="H1026" s="14"/>
       <c r="I1026" s="2"/>
       <c r="K1026" s="2"/>
     </row>
@@ -25424,7 +25647,7 @@
       <c r="C1027" s="2"/>
       <c r="D1027" s="2"/>
       <c r="G1027" s="2"/>
-      <c r="H1027" s="15"/>
+      <c r="H1027" s="14"/>
       <c r="I1027" s="2"/>
       <c r="K1027" s="2"/>
     </row>
@@ -25434,7 +25657,7 @@
       <c r="C1028" s="2"/>
       <c r="D1028" s="2"/>
       <c r="G1028" s="2"/>
-      <c r="H1028" s="15"/>
+      <c r="H1028" s="14"/>
       <c r="I1028" s="2"/>
       <c r="K1028" s="2"/>
     </row>
@@ -25444,7 +25667,7 @@
       <c r="C1029" s="2"/>
       <c r="D1029" s="2"/>
       <c r="G1029" s="2"/>
-      <c r="H1029" s="15"/>
+      <c r="H1029" s="14"/>
       <c r="I1029" s="2"/>
       <c r="K1029" s="2"/>
     </row>
@@ -25454,7 +25677,7 @@
       <c r="C1030" s="2"/>
       <c r="D1030" s="2"/>
       <c r="G1030" s="2"/>
-      <c r="H1030" s="15"/>
+      <c r="H1030" s="14"/>
       <c r="I1030" s="2"/>
       <c r="K1030" s="2"/>
     </row>
@@ -25464,7 +25687,7 @@
       <c r="C1031" s="2"/>
       <c r="D1031" s="2"/>
       <c r="G1031" s="2"/>
-      <c r="H1031" s="15"/>
+      <c r="H1031" s="14"/>
       <c r="I1031" s="2"/>
       <c r="K1031" s="2"/>
     </row>
@@ -25474,7 +25697,7 @@
       <c r="C1032" s="2"/>
       <c r="D1032" s="2"/>
       <c r="G1032" s="2"/>
-      <c r="H1032" s="15"/>
+      <c r="H1032" s="14"/>
       <c r="I1032" s="2"/>
       <c r="K1032" s="2"/>
     </row>
@@ -25484,7 +25707,7 @@
       <c r="C1033" s="2"/>
       <c r="D1033" s="2"/>
       <c r="G1033" s="2"/>
-      <c r="H1033" s="15"/>
+      <c r="H1033" s="14"/>
       <c r="I1033" s="2"/>
       <c r="K1033" s="2"/>
     </row>
@@ -25494,7 +25717,7 @@
       <c r="C1034" s="2"/>
       <c r="D1034" s="2"/>
       <c r="G1034" s="2"/>
-      <c r="H1034" s="15"/>
+      <c r="H1034" s="14"/>
       <c r="I1034" s="2"/>
       <c r="K1034" s="2"/>
     </row>
@@ -25504,7 +25727,7 @@
       <c r="C1035" s="2"/>
       <c r="D1035" s="2"/>
       <c r="G1035" s="2"/>
-      <c r="H1035" s="15"/>
+      <c r="H1035" s="14"/>
       <c r="I1035" s="2"/>
       <c r="K1035" s="2"/>
     </row>
@@ -25514,7 +25737,7 @@
       <c r="C1036" s="2"/>
       <c r="D1036" s="2"/>
       <c r="G1036" s="2"/>
-      <c r="H1036" s="15"/>
+      <c r="H1036" s="14"/>
       <c r="I1036" s="2"/>
       <c r="K1036" s="2"/>
     </row>
@@ -25524,7 +25747,7 @@
       <c r="C1037" s="2"/>
       <c r="D1037" s="2"/>
       <c r="G1037" s="2"/>
-      <c r="H1037" s="15"/>
+      <c r="H1037" s="14"/>
       <c r="I1037" s="2"/>
       <c r="K1037" s="2"/>
     </row>
@@ -25534,7 +25757,7 @@
       <c r="C1038" s="2"/>
       <c r="D1038" s="2"/>
       <c r="G1038" s="2"/>
-      <c r="H1038" s="15"/>
+      <c r="H1038" s="14"/>
       <c r="I1038" s="2"/>
       <c r="K1038" s="2"/>
     </row>
@@ -25544,7 +25767,7 @@
       <c r="C1039" s="2"/>
       <c r="D1039" s="2"/>
       <c r="G1039" s="2"/>
-      <c r="H1039" s="15"/>
+      <c r="H1039" s="14"/>
       <c r="I1039" s="2"/>
       <c r="K1039" s="2"/>
     </row>
@@ -25554,7 +25777,7 @@
       <c r="C1040" s="2"/>
       <c r="D1040" s="2"/>
       <c r="G1040" s="2"/>
-      <c r="H1040" s="15"/>
+      <c r="H1040" s="14"/>
       <c r="I1040" s="2"/>
       <c r="K1040" s="2"/>
     </row>
@@ -25564,7 +25787,7 @@
       <c r="C1041" s="2"/>
       <c r="D1041" s="2"/>
       <c r="G1041" s="2"/>
-      <c r="H1041" s="15"/>
+      <c r="H1041" s="14"/>
       <c r="I1041" s="2"/>
       <c r="K1041" s="2"/>
     </row>
@@ -25574,7 +25797,7 @@
       <c r="C1042" s="2"/>
       <c r="D1042" s="2"/>
       <c r="G1042" s="2"/>
-      <c r="H1042" s="15"/>
+      <c r="H1042" s="14"/>
       <c r="I1042" s="2"/>
       <c r="K1042" s="2"/>
     </row>
@@ -25584,7 +25807,7 @@
       <c r="C1043" s="2"/>
       <c r="D1043" s="2"/>
       <c r="G1043" s="2"/>
-      <c r="H1043" s="15"/>
+      <c r="H1043" s="14"/>
       <c r="I1043" s="2"/>
       <c r="K1043" s="2"/>
     </row>
@@ -25594,7 +25817,7 @@
       <c r="C1044" s="2"/>
       <c r="D1044" s="2"/>
       <c r="G1044" s="2"/>
-      <c r="H1044" s="15"/>
+      <c r="H1044" s="14"/>
       <c r="I1044" s="2"/>
       <c r="K1044" s="2"/>
     </row>
@@ -25604,7 +25827,7 @@
       <c r="C1045" s="2"/>
       <c r="D1045" s="2"/>
       <c r="G1045" s="2"/>
-      <c r="H1045" s="15"/>
+      <c r="H1045" s="14"/>
       <c r="I1045" s="2"/>
       <c r="K1045" s="2"/>
     </row>
@@ -25614,7 +25837,7 @@
       <c r="C1046" s="2"/>
       <c r="D1046" s="2"/>
       <c r="G1046" s="2"/>
-      <c r="H1046" s="15"/>
+      <c r="H1046" s="14"/>
       <c r="I1046" s="2"/>
       <c r="K1046" s="2"/>
     </row>
@@ -25624,7 +25847,7 @@
       <c r="C1047" s="2"/>
       <c r="D1047" s="2"/>
       <c r="G1047" s="2"/>
-      <c r="H1047" s="15"/>
+      <c r="H1047" s="14"/>
       <c r="I1047" s="2"/>
       <c r="K1047" s="2"/>
     </row>
@@ -25634,7 +25857,7 @@
       <c r="C1048" s="2"/>
       <c r="D1048" s="2"/>
       <c r="G1048" s="2"/>
-      <c r="H1048" s="15"/>
+      <c r="H1048" s="14"/>
       <c r="I1048" s="2"/>
       <c r="K1048" s="2"/>
     </row>
@@ -25644,7 +25867,7 @@
       <c r="C1049" s="2"/>
       <c r="D1049" s="2"/>
       <c r="G1049" s="2"/>
-      <c r="H1049" s="15"/>
+      <c r="H1049" s="14"/>
       <c r="I1049" s="2"/>
       <c r="K1049" s="2"/>
     </row>
@@ -25654,7 +25877,7 @@
       <c r="C1050" s="2"/>
       <c r="D1050" s="2"/>
       <c r="G1050" s="2"/>
-      <c r="H1050" s="15"/>
+      <c r="H1050" s="14"/>
       <c r="I1050" s="2"/>
       <c r="K1050" s="2"/>
     </row>
@@ -25664,7 +25887,7 @@
       <c r="C1051" s="2"/>
       <c r="D1051" s="2"/>
       <c r="G1051" s="2"/>
-      <c r="H1051" s="15"/>
+      <c r="H1051" s="14"/>
       <c r="I1051" s="2"/>
       <c r="K1051" s="2"/>
     </row>
@@ -25674,7 +25897,7 @@
       <c r="C1052" s="2"/>
       <c r="D1052" s="2"/>
       <c r="G1052" s="2"/>
-      <c r="H1052" s="15"/>
+      <c r="H1052" s="14"/>
       <c r="I1052" s="2"/>
       <c r="K1052" s="2"/>
     </row>
@@ -25684,7 +25907,7 @@
       <c r="C1053" s="2"/>
       <c r="D1053" s="2"/>
       <c r="G1053" s="2"/>
-      <c r="H1053" s="15"/>
+      <c r="H1053" s="14"/>
       <c r="I1053" s="2"/>
       <c r="K1053" s="2"/>
     </row>
@@ -25694,7 +25917,7 @@
       <c r="C1054" s="2"/>
       <c r="D1054" s="2"/>
       <c r="G1054" s="2"/>
-      <c r="H1054" s="15"/>
+      <c r="H1054" s="14"/>
       <c r="I1054" s="2"/>
       <c r="K1054" s="2"/>
     </row>
@@ -25704,7 +25927,7 @@
       <c r="C1055" s="2"/>
       <c r="D1055" s="2"/>
       <c r="G1055" s="2"/>
-      <c r="H1055" s="15"/>
+      <c r="H1055" s="14"/>
       <c r="I1055" s="2"/>
       <c r="K1055" s="2"/>
     </row>
@@ -25714,7 +25937,7 @@
       <c r="C1056" s="2"/>
       <c r="D1056" s="2"/>
       <c r="G1056" s="2"/>
-      <c r="H1056" s="15"/>
+      <c r="H1056" s="14"/>
       <c r="I1056" s="2"/>
       <c r="K1056" s="2"/>
     </row>
@@ -25724,7 +25947,7 @@
       <c r="C1057" s="2"/>
       <c r="D1057" s="2"/>
       <c r="G1057" s="2"/>
-      <c r="H1057" s="15"/>
+      <c r="H1057" s="14"/>
       <c r="I1057" s="2"/>
       <c r="K1057" s="2"/>
     </row>
@@ -25734,7 +25957,7 @@
       <c r="C1058" s="2"/>
       <c r="D1058" s="2"/>
       <c r="G1058" s="2"/>
-      <c r="H1058" s="15"/>
+      <c r="H1058" s="14"/>
       <c r="I1058" s="2"/>
       <c r="K1058" s="2"/>
     </row>
@@ -25744,7 +25967,7 @@
       <c r="C1059" s="2"/>
       <c r="D1059" s="2"/>
       <c r="G1059" s="2"/>
-      <c r="H1059" s="15"/>
+      <c r="H1059" s="14"/>
       <c r="I1059" s="2"/>
       <c r="K1059" s="2"/>
     </row>
@@ -25754,7 +25977,7 @@
       <c r="C1060" s="2"/>
       <c r="D1060" s="2"/>
       <c r="G1060" s="2"/>
-      <c r="H1060" s="15"/>
+      <c r="H1060" s="14"/>
       <c r="I1060" s="2"/>
       <c r="K1060" s="2"/>
     </row>
@@ -25764,7 +25987,7 @@
       <c r="C1061" s="2"/>
       <c r="D1061" s="2"/>
       <c r="G1061" s="2"/>
-      <c r="H1061" s="15"/>
+      <c r="H1061" s="14"/>
       <c r="I1061" s="2"/>
       <c r="K1061" s="2"/>
     </row>
@@ -25774,7 +25997,7 @@
       <c r="C1062" s="2"/>
       <c r="D1062" s="2"/>
       <c r="G1062" s="2"/>
-      <c r="H1062" s="15"/>
+      <c r="H1062" s="14"/>
       <c r="I1062" s="2"/>
       <c r="K1062" s="2"/>
     </row>
@@ -25784,7 +26007,7 @@
       <c r="C1063" s="2"/>
       <c r="D1063" s="2"/>
       <c r="G1063" s="2"/>
-      <c r="H1063" s="15"/>
+      <c r="H1063" s="14"/>
       <c r="I1063" s="2"/>
       <c r="K1063" s="2"/>
     </row>
@@ -25794,7 +26017,7 @@
       <c r="C1064" s="2"/>
       <c r="D1064" s="2"/>
       <c r="G1064" s="2"/>
-      <c r="H1064" s="15"/>
+      <c r="H1064" s="14"/>
       <c r="I1064" s="2"/>
       <c r="K1064" s="2"/>
     </row>
@@ -25833,14 +26056,56 @@
     <hyperlink ref="D240" r:id="rId31" display="imagenes\espana-2012-unesco-burgos .jpg" xr:uid="{77F7290A-D8B4-4A53-B6CB-B7C4AFEE476C}"/>
     <hyperlink ref="D239" r:id="rId32" display="imagenes\espana-2011-unesco-granada..jpg" xr:uid="{7FA02833-6422-4849-AD6F-38D1F2A3A402}"/>
     <hyperlink ref="D238" r:id="rId33" display="imagenes\espana-2010-unesco-cordoba.jpg" xr:uid="{BEDF9C40-C842-4772-B62A-B5B23756D4A7}"/>
+    <hyperlink ref="D43" r:id="rId34" xr:uid="{C75600DE-F7BC-4388-925F-3B565C259F0C}"/>
+    <hyperlink ref="D2" r:id="rId35" display="imagenes\alemania-2006-schleswig-holstein.jpg" xr:uid="{D9CC799D-EE35-4ED3-8388-6C2C4082966A}"/>
+    <hyperlink ref="D3" r:id="rId36" display="imagenes\alemania-2007-pomerania-occidental.jpg" xr:uid="{8083EA68-3045-4997-A889-05999632F1DC}"/>
+    <hyperlink ref="D4" r:id="rId37" display="imagenes\alemania-2007-tratado-roma.jpg" xr:uid="{D8D78FC9-44CC-4C0C-93AB-74ACCA7A50DA}"/>
+    <hyperlink ref="D5" r:id="rId38" display="imagenes\alemania-2008-hamburgo.jpg" xr:uid="{6F8D23C4-B962-43BD-B106-E3A45E934E34}"/>
+    <hyperlink ref="D6" r:id="rId39" display="imagenes\alemania-2009-aniversario-union-economica.jpg" xr:uid="{D7DFC79E-FFB8-4D7D-8ACF-7FE721763639}"/>
+    <hyperlink ref="D7" r:id="rId40" display="imagenes\alemania-2009-Sarre.jpg" xr:uid="{D528F2A3-8EFB-4975-894B-A1C0CEA13839}"/>
+    <hyperlink ref="D8" r:id="rId41" display="imagenes\alemania-2010-bremen.jpg" xr:uid="{AC57C239-81CB-44C4-B2D5-7B2791BFB9C7}"/>
+    <hyperlink ref="D9" r:id="rId42" display="imagenes\alemania-2011-renania-westfalia.jpg" xr:uid="{F584B395-D71B-4660-B443-8E4335E37E43}"/>
+    <hyperlink ref="D10" r:id="rId43" display="imagenes\alemania-2012-baviera.jpg" xr:uid="{048F328F-0352-4084-9267-B0E748902A28}"/>
+    <hyperlink ref="D11" r:id="rId44" display="imagenes\alemania-2012-10anios-billetes-monedas-euros.jpg" xr:uid="{D33F8553-C21F-4270-AC52-01A75A89F24B}"/>
+    <hyperlink ref="D12" r:id="rId45" display="imagenes\alemania-2013-tratado-eliseo.jpg" xr:uid="{895C6E2C-FD31-4B54-A2FC-74A2FE0DCB29}"/>
+    <hyperlink ref="D13" r:id="rId46" display="imagenes\alemania-2013-baden-wurttemberg .jpg" xr:uid="{E8E086E1-4228-4AEC-A565-4263A088977D}"/>
+    <hyperlink ref="D14" r:id="rId47" display="imagenes\alemania-2014-baja-sajonia.jpg" xr:uid="{54FDE33B-AA52-4421-99B0-5DF90D07EE7A}"/>
+    <hyperlink ref="D15" r:id="rId48" display="imagenes\alemania-2015-hesse.jpg" xr:uid="{FCA4FFB9-E3B4-4414-A843-2398793812CA}"/>
+    <hyperlink ref="D16" r:id="rId49" display="imagenes\alemania-2015-unidad-alemana.jpg" xr:uid="{F55E7389-EA67-43C3-A647-838664AA6374}"/>
+    <hyperlink ref="D17" r:id="rId50" display="imagenes\alemania-2015-aniversario-bandera-ue.jpg" xr:uid="{AA3FEFC6-4015-4A86-9CC4-3E5468F5A907}"/>
+    <hyperlink ref="D18" r:id="rId51" display="imagenes\alemania-2016-sajonia.jpg" xr:uid="{0A028D22-9A3D-49FC-BDD9-58174323A1AB}"/>
+    <hyperlink ref="D19" r:id="rId52" display="imagenes\alemania-2017-renania-palatinado.jpg" xr:uid="{DCD0874E-3A35-4B80-B04E-3B4835E0E5EA}"/>
+    <hyperlink ref="D20" r:id="rId53" display="imagenes\alemania-2018-berlín.jpg" xr:uid="{C441EBAC-4E6F-4845-8859-F16B7D4C8412}"/>
+    <hyperlink ref="D21" r:id="rId54" display="imagenes\alemania-2018-helmut-schmidt.jpg" xr:uid="{4C03DFDD-9A39-40C7-BBAE-0A1FD0A04C6D}"/>
+    <hyperlink ref="D22" r:id="rId55" display="imagenes\alemania-2019-bundesrat..jpg" xr:uid="{0560FF2E-D22A-413E-BAA3-35E03ABA9979}"/>
+    <hyperlink ref="D23" r:id="rId56" display="imagenes\alemania-2019-caida-muro-berlin.jpg" xr:uid="{0F5D7EBC-EE7E-46BA-AFAF-7F2AA9727F0F}"/>
+    <hyperlink ref="D24" r:id="rId57" display="imagenes\alemania-2020-brandeburgo.jpg" xr:uid="{EC37AD67-A1D6-47ED-95E6-5F19F0B97764}"/>
+    <hyperlink ref="D25" r:id="rId58" display="imagenes\alemania-2020-arrodillamiento-varsovia.jpg" xr:uid="{76C0B07A-7BDC-4319-ABD3-B88E4F745AD5}"/>
+    <hyperlink ref="D26" r:id="rId59" display="imagenes\alemania-2021-sajonia-anhalt .jpg" xr:uid="{B3001A05-971C-4D36-A2E2-9F8A21351779}"/>
+    <hyperlink ref="D28" r:id="rId60" display="imagenes\alemania-2022-erasmus.jpg" xr:uid="{5ECA9298-CEC3-4AA7-AF96-457FD2828E0A}"/>
+    <hyperlink ref="D27" r:id="rId61" display="imagenes\alemania-2022-turingia.jpg" xr:uid="{38DC0DC2-B386-49C8-A4E5-5DBA4B1BF52E}"/>
+    <hyperlink ref="D29" r:id="rId62" display="imagenes\alemania-2023-hamburgo.jpg" xr:uid="{FAACB0FE-1B31-4046-8394-F94CFBB8A6AA}"/>
+    <hyperlink ref="D30" r:id="rId63" display="imagenes\alemania-2023-carlomagno.jpg" xr:uid="{C20CFE1A-C09C-4620-B7EA-43385E156560}"/>
+    <hyperlink ref="D31" r:id="rId64" display="imagenes\alemania-2024-pomerania-occidental.jpg" xr:uid="{159422B5-CB79-4614-9401-DDE56501F37C}"/>
+    <hyperlink ref="D32" r:id="rId65" display="imagenes\alemania-2024-constitución-paulskirche.jpg" xr:uid="{2A92E3FB-8DF7-4021-817B-9F38A329C5CA}"/>
+    <hyperlink ref="D33" r:id="rId66" display="imagenes\alemania-2025-reunificación-alemania.jpg" xr:uid="{8BCD5398-A07A-4C75-B488-4B47E87D62A1}"/>
+    <hyperlink ref="D34" r:id="rId67" display="imagenes\alemania-2025-sarre.jpg" xr:uid="{1FB1BC55-C8D4-4A39-858A-D4F514C867DC}"/>
+    <hyperlink ref="D35" r:id="rId68" display="imagenes\alemania-2026-bremen.jpg" xr:uid="{E42A437E-2F02-4936-AABF-EEC937F521A5}"/>
+    <hyperlink ref="D36" r:id="rId69" display="imagenes\alemania-2026-konrad-adenauer.jpg" xr:uid="{056A136A-DAAE-44A2-A61E-BDD70C3278EA}"/>
+    <hyperlink ref="D37" r:id="rId70" display="imagenes\alemania-2027-renania-westfalia.jpg" xr:uid="{818D09FB-4DD5-4774-AA47-4C72349B861F}"/>
+    <hyperlink ref="D38" r:id="rId71" display="imagenes\alemania-2027-dietrich-genscher.jpg" xr:uid="{6D8E9067-C43D-461A-A648-595655BFE0D3}"/>
+    <hyperlink ref="D39" r:id="rId72" display="imagenes\alemania-2028-richard-von-weizsacker.jpg" xr:uid="{F7C51BB6-840B-4713-87C0-9B309366D75E}"/>
+    <hyperlink ref="D40" r:id="rId73" display="imagenes\alemania-2029-annemarie-renger.jpg" xr:uid="{74A39BE8-7C43-401F-98E9-8C39C621D910}"/>
+    <hyperlink ref="D41" r:id="rId74" display="imagenes\alemania-2030-helmut-kohl.jpg" xr:uid="{1242EF6E-7232-4799-81AE-3D20E6B769DF}"/>
+    <hyperlink ref="D42" r:id="rId75" display="imagenes\alemania-2031-regine-hildebrandt.jpg" xr:uid="{EF0C9890-F8AB-40C0-8C81-C3651B1C3D8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId76"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="7" man="1"/>
   </colBreaks>
   <tableParts count="1">
-    <tablePart r:id="rId34"/>
+    <tablePart r:id="rId77"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>